<commit_message>
Add emergency contact relationship
</commit_message>
<xml_diff>
--- a/erp-v2/assets/templates/employee-import-template.xlsx
+++ b/erp-v2/assets/templates/employee-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="員工匯入範本" sheetId="1" r:id="Rdc8c0bfe81d840c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填寫說明" sheetId="2" r:id="R1bbb67a824a54ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="員工匯入範本" sheetId="1" r:id="R08863dd0515e47ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填寫說明" sheetId="2" r:id="R5c5a39db11ba4764"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,9 +14,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
-  </x:numFmts>
   <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
@@ -119,7 +116,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="29">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -175,9 +172,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -390,149 +384,48 @@
     <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="15" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="13" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="14" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="15" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="13" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="16" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="15" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="13" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="15" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="17" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="13" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="20" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="15" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="17" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="13" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="20" hidden="0" customWidth="1"/>
-    <x:col min="28" max="28" width="15" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="20" hidden="0" customWidth="1"/>
     <x:col min="29" max="29" width="15" hidden="0" customWidth="1"/>
     <x:col min="30" max="30" width="15" hidden="0" customWidth="1"/>
     <x:col min="31" max="31" width="15" hidden="0" customWidth="1"/>
-    <x:col min="32" max="32" width="17" hidden="0" customWidth="1"/>
-    <x:col min="33" max="33" width="16" hidden="0" customWidth="1"/>
-    <x:col min="34" max="34" width="28" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="15" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="17" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="16" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>紘嘉物業 ERP｜員工資料批次匯入範本</x:v>
       </x:c>
-      <x:c r="B1"/>
-      <x:c r="C1"/>
-      <x:c r="D1"/>
-      <x:c r="E1"/>
-      <x:c r="F1"/>
-      <x:c r="G1"/>
-      <x:c r="H1"/>
-      <x:c r="I1"/>
-      <x:c r="J1"/>
-      <x:c r="K1"/>
-      <x:c r="L1"/>
-      <x:c r="M1"/>
-      <x:c r="N1"/>
-      <x:c r="O1"/>
-      <x:c r="P1"/>
-      <x:c r="Q1"/>
-      <x:c r="R1"/>
-      <x:c r="S1"/>
-      <x:c r="T1"/>
-      <x:c r="U1"/>
-      <x:c r="V1"/>
-      <x:c r="W1"/>
-      <x:c r="X1"/>
-      <x:c r="Y1"/>
-      <x:c r="Z1"/>
-      <x:c r="AA1"/>
-      <x:c r="AB1"/>
-      <x:c r="AC1"/>
-      <x:c r="AD1"/>
-      <x:c r="AE1"/>
-      <x:c r="AF1"/>
-      <x:c r="AG1"/>
-      <x:c r="AH1"/>
-      <x:c r="AI1"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="9" t="str">
         <x:v>請從第 5 列開始填寫；「工號、姓名」為必填。日期使用 YYYY-MM-DD。初始密碼留空就不建立／變更登入帳號。請勿刪除或更名標題列。</x:v>
       </x:c>
-      <x:c r="B2"/>
-      <x:c r="C2"/>
-      <x:c r="D2"/>
-      <x:c r="E2"/>
-      <x:c r="F2"/>
-      <x:c r="G2"/>
-      <x:c r="H2"/>
-      <x:c r="I2"/>
-      <x:c r="J2"/>
-      <x:c r="K2"/>
-      <x:c r="L2"/>
-      <x:c r="M2"/>
-      <x:c r="N2"/>
-      <x:c r="O2"/>
-      <x:c r="P2"/>
-      <x:c r="Q2"/>
-      <x:c r="R2"/>
-      <x:c r="S2"/>
-      <x:c r="T2"/>
-      <x:c r="U2"/>
-      <x:c r="V2"/>
-      <x:c r="W2"/>
-      <x:c r="X2"/>
-      <x:c r="Y2"/>
-      <x:c r="Z2"/>
-      <x:c r="AA2"/>
-      <x:c r="AB2"/>
-      <x:c r="AC2"/>
-      <x:c r="AD2"/>
-      <x:c r="AE2"/>
-      <x:c r="AF2"/>
-      <x:c r="AG2"/>
-      <x:c r="AH2"/>
-      <x:c r="AI2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11" t="str">
         <x:v>可一次貼上或填寫多位員工；上傳後 ERP 會先顯示預覽與錯誤，再由您確認批次新增或依工號更新。</x:v>
       </x:c>
-      <x:c r="B3"/>
-      <x:c r="C3"/>
-      <x:c r="D3"/>
-      <x:c r="E3"/>
-      <x:c r="F3"/>
-      <x:c r="G3"/>
-      <x:c r="H3"/>
-      <x:c r="I3"/>
-      <x:c r="J3"/>
-      <x:c r="K3"/>
-      <x:c r="L3"/>
-      <x:c r="M3"/>
-      <x:c r="N3"/>
-      <x:c r="O3"/>
-      <x:c r="P3"/>
-      <x:c r="Q3"/>
-      <x:c r="R3"/>
-      <x:c r="S3"/>
-      <x:c r="T3"/>
-      <x:c r="U3"/>
-      <x:c r="V3"/>
-      <x:c r="W3"/>
-      <x:c r="X3"/>
-      <x:c r="Y3"/>
-      <x:c r="Z3"/>
-      <x:c r="AA3"/>
-      <x:c r="AB3"/>
-      <x:c r="AC3"/>
-      <x:c r="AD3"/>
-      <x:c r="AE3"/>
-      <x:c r="AF3"/>
-      <x:c r="AG3"/>
-      <x:c r="AH3"/>
-      <x:c r="AI3"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="17" t="str">
@@ -563,16 +456,16 @@
         <x:v>身分證字號</x:v>
       </x:c>
       <x:c r="J4" s="17" t="str">
-        <x:v>出生年月日</x:v>
+        <x:v>戶籍地址</x:v>
       </x:c>
       <x:c r="K4" s="17" t="str">
-        <x:v>戶籍地址</x:v>
+        <x:v>現居地址</x:v>
       </x:c>
       <x:c r="L4" s="17" t="str">
-        <x:v>現居地址</x:v>
+        <x:v>緊急聯絡人</x:v>
       </x:c>
       <x:c r="M4" s="17" t="str">
-        <x:v>緊急聯絡人</x:v>
+        <x:v>緊急聯絡人關係</x:v>
       </x:c>
       <x:c r="N4" s="17" t="str">
         <x:v>緊急聯絡電話</x:v>
@@ -637,7 +530,7 @@
       <x:c r="AH4" s="17" t="str">
         <x:v>薪資生效日期</x:v>
       </x:c>
-      <x:c r="AI4" t="str">
+      <x:c r="AI4" s="17" t="str">
         <x:v>可排班案場</x:v>
       </x:c>
     </x:row>
@@ -651,7 +544,7 @@
       <x:c r="G5" s="21"/>
       <x:c r="H5" s="21"/>
       <x:c r="I5" s="21"/>
-      <x:c r="J5" s="28"/>
+      <x:c r="J5" s="21"/>
       <x:c r="K5" s="21"/>
       <x:c r="L5" s="21"/>
       <x:c r="M5" s="21"/>
@@ -676,7 +569,7 @@
       <x:c r="AF5" s="21"/>
       <x:c r="AG5" s="21"/>
       <x:c r="AH5" s="21"/>
-      <x:c r="AI5"/>
+      <x:c r="AI5" s="21"/>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="21"/>
@@ -688,7 +581,7 @@
       <x:c r="G6" s="21"/>
       <x:c r="H6" s="21"/>
       <x:c r="I6" s="21"/>
-      <x:c r="J6" s="28"/>
+      <x:c r="J6" s="21"/>
       <x:c r="K6" s="21"/>
       <x:c r="L6" s="21"/>
       <x:c r="M6" s="21"/>
@@ -713,7 +606,7 @@
       <x:c r="AF6" s="21"/>
       <x:c r="AG6" s="21"/>
       <x:c r="AH6" s="21"/>
-      <x:c r="AI6"/>
+      <x:c r="AI6" s="21"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="21"/>
@@ -725,7 +618,7 @@
       <x:c r="G7" s="21"/>
       <x:c r="H7" s="21"/>
       <x:c r="I7" s="21"/>
-      <x:c r="J7" s="28"/>
+      <x:c r="J7" s="21"/>
       <x:c r="K7" s="21"/>
       <x:c r="L7" s="21"/>
       <x:c r="M7" s="21"/>
@@ -750,7 +643,7 @@
       <x:c r="AF7" s="21"/>
       <x:c r="AG7" s="21"/>
       <x:c r="AH7" s="21"/>
-      <x:c r="AI7"/>
+      <x:c r="AI7" s="21"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="21"/>
@@ -762,7 +655,7 @@
       <x:c r="G8" s="21"/>
       <x:c r="H8" s="21"/>
       <x:c r="I8" s="21"/>
-      <x:c r="J8" s="28"/>
+      <x:c r="J8" s="21"/>
       <x:c r="K8" s="21"/>
       <x:c r="L8" s="21"/>
       <x:c r="M8" s="21"/>
@@ -787,7 +680,7 @@
       <x:c r="AF8" s="21"/>
       <x:c r="AG8" s="21"/>
       <x:c r="AH8" s="21"/>
-      <x:c r="AI8"/>
+      <x:c r="AI8" s="21"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="21"/>
@@ -799,7 +692,7 @@
       <x:c r="G9" s="21"/>
       <x:c r="H9" s="21"/>
       <x:c r="I9" s="21"/>
-      <x:c r="J9" s="28"/>
+      <x:c r="J9" s="21"/>
       <x:c r="K9" s="21"/>
       <x:c r="L9" s="21"/>
       <x:c r="M9" s="21"/>
@@ -824,7 +717,7 @@
       <x:c r="AF9" s="21"/>
       <x:c r="AG9" s="21"/>
       <x:c r="AH9" s="21"/>
-      <x:c r="AI9"/>
+      <x:c r="AI9" s="21"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="21"/>
@@ -836,7 +729,7 @@
       <x:c r="G10" s="21"/>
       <x:c r="H10" s="21"/>
       <x:c r="I10" s="21"/>
-      <x:c r="J10" s="28"/>
+      <x:c r="J10" s="21"/>
       <x:c r="K10" s="21"/>
       <x:c r="L10" s="21"/>
       <x:c r="M10" s="21"/>
@@ -861,7 +754,7 @@
       <x:c r="AF10" s="21"/>
       <x:c r="AG10" s="21"/>
       <x:c r="AH10" s="21"/>
-      <x:c r="AI10"/>
+      <x:c r="AI10" s="21"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="21"/>
@@ -873,7 +766,7 @@
       <x:c r="G11" s="21"/>
       <x:c r="H11" s="21"/>
       <x:c r="I11" s="21"/>
-      <x:c r="J11" s="28"/>
+      <x:c r="J11" s="21"/>
       <x:c r="K11" s="21"/>
       <x:c r="L11" s="21"/>
       <x:c r="M11" s="21"/>
@@ -898,7 +791,7 @@
       <x:c r="AF11" s="21"/>
       <x:c r="AG11" s="21"/>
       <x:c r="AH11" s="21"/>
-      <x:c r="AI11"/>
+      <x:c r="AI11" s="21"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="21"/>
@@ -910,7 +803,7 @@
       <x:c r="G12" s="21"/>
       <x:c r="H12" s="21"/>
       <x:c r="I12" s="21"/>
-      <x:c r="J12" s="28"/>
+      <x:c r="J12" s="21"/>
       <x:c r="K12" s="21"/>
       <x:c r="L12" s="21"/>
       <x:c r="M12" s="21"/>
@@ -935,7 +828,7 @@
       <x:c r="AF12" s="21"/>
       <x:c r="AG12" s="21"/>
       <x:c r="AH12" s="21"/>
-      <x:c r="AI12"/>
+      <x:c r="AI12" s="21"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="21"/>
@@ -947,7 +840,7 @@
       <x:c r="G13" s="21"/>
       <x:c r="H13" s="21"/>
       <x:c r="I13" s="21"/>
-      <x:c r="J13" s="28"/>
+      <x:c r="J13" s="21"/>
       <x:c r="K13" s="21"/>
       <x:c r="L13" s="21"/>
       <x:c r="M13" s="21"/>
@@ -972,7 +865,7 @@
       <x:c r="AF13" s="21"/>
       <x:c r="AG13" s="21"/>
       <x:c r="AH13" s="21"/>
-      <x:c r="AI13"/>
+      <x:c r="AI13" s="21"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="21"/>
@@ -984,7 +877,7 @@
       <x:c r="G14" s="21"/>
       <x:c r="H14" s="21"/>
       <x:c r="I14" s="21"/>
-      <x:c r="J14" s="28"/>
+      <x:c r="J14" s="21"/>
       <x:c r="K14" s="21"/>
       <x:c r="L14" s="21"/>
       <x:c r="M14" s="21"/>
@@ -1009,7 +902,7 @@
       <x:c r="AF14" s="21"/>
       <x:c r="AG14" s="21"/>
       <x:c r="AH14" s="21"/>
-      <x:c r="AI14"/>
+      <x:c r="AI14" s="21"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="21"/>
@@ -1021,7 +914,7 @@
       <x:c r="G15" s="21"/>
       <x:c r="H15" s="21"/>
       <x:c r="I15" s="21"/>
-      <x:c r="J15" s="28"/>
+      <x:c r="J15" s="21"/>
       <x:c r="K15" s="21"/>
       <x:c r="L15" s="21"/>
       <x:c r="M15" s="21"/>
@@ -1046,7 +939,7 @@
       <x:c r="AF15" s="21"/>
       <x:c r="AG15" s="21"/>
       <x:c r="AH15" s="21"/>
-      <x:c r="AI15"/>
+      <x:c r="AI15" s="21"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="21"/>
@@ -1058,7 +951,7 @@
       <x:c r="G16" s="21"/>
       <x:c r="H16" s="21"/>
       <x:c r="I16" s="21"/>
-      <x:c r="J16" s="28"/>
+      <x:c r="J16" s="21"/>
       <x:c r="K16" s="21"/>
       <x:c r="L16" s="21"/>
       <x:c r="M16" s="21"/>
@@ -1083,7 +976,7 @@
       <x:c r="AF16" s="21"/>
       <x:c r="AG16" s="21"/>
       <x:c r="AH16" s="21"/>
-      <x:c r="AI16"/>
+      <x:c r="AI16" s="21"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="21"/>
@@ -1095,7 +988,7 @@
       <x:c r="G17" s="21"/>
       <x:c r="H17" s="21"/>
       <x:c r="I17" s="21"/>
-      <x:c r="J17" s="28"/>
+      <x:c r="J17" s="21"/>
       <x:c r="K17" s="21"/>
       <x:c r="L17" s="21"/>
       <x:c r="M17" s="21"/>
@@ -1120,7 +1013,7 @@
       <x:c r="AF17" s="21"/>
       <x:c r="AG17" s="21"/>
       <x:c r="AH17" s="21"/>
-      <x:c r="AI17"/>
+      <x:c r="AI17" s="21"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="21"/>
@@ -1132,7 +1025,7 @@
       <x:c r="G18" s="21"/>
       <x:c r="H18" s="21"/>
       <x:c r="I18" s="21"/>
-      <x:c r="J18" s="28"/>
+      <x:c r="J18" s="21"/>
       <x:c r="K18" s="21"/>
       <x:c r="L18" s="21"/>
       <x:c r="M18" s="21"/>
@@ -1157,7 +1050,7 @@
       <x:c r="AF18" s="21"/>
       <x:c r="AG18" s="21"/>
       <x:c r="AH18" s="21"/>
-      <x:c r="AI18"/>
+      <x:c r="AI18" s="21"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="21"/>
@@ -1169,7 +1062,7 @@
       <x:c r="G19" s="21"/>
       <x:c r="H19" s="21"/>
       <x:c r="I19" s="21"/>
-      <x:c r="J19" s="28"/>
+      <x:c r="J19" s="21"/>
       <x:c r="K19" s="21"/>
       <x:c r="L19" s="21"/>
       <x:c r="M19" s="21"/>
@@ -1194,7 +1087,7 @@
       <x:c r="AF19" s="21"/>
       <x:c r="AG19" s="21"/>
       <x:c r="AH19" s="21"/>
-      <x:c r="AI19"/>
+      <x:c r="AI19" s="21"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="21"/>
@@ -1206,7 +1099,7 @@
       <x:c r="G20" s="21"/>
       <x:c r="H20" s="21"/>
       <x:c r="I20" s="21"/>
-      <x:c r="J20" s="28"/>
+      <x:c r="J20" s="21"/>
       <x:c r="K20" s="21"/>
       <x:c r="L20" s="21"/>
       <x:c r="M20" s="21"/>
@@ -1231,7 +1124,7 @@
       <x:c r="AF20" s="21"/>
       <x:c r="AG20" s="21"/>
       <x:c r="AH20" s="21"/>
-      <x:c r="AI20"/>
+      <x:c r="AI20" s="21"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="21"/>
@@ -1243,7 +1136,7 @@
       <x:c r="G21" s="21"/>
       <x:c r="H21" s="21"/>
       <x:c r="I21" s="21"/>
-      <x:c r="J21" s="28"/>
+      <x:c r="J21" s="21"/>
       <x:c r="K21" s="21"/>
       <x:c r="L21" s="21"/>
       <x:c r="M21" s="21"/>
@@ -1268,7 +1161,7 @@
       <x:c r="AF21" s="21"/>
       <x:c r="AG21" s="21"/>
       <x:c r="AH21" s="21"/>
-      <x:c r="AI21"/>
+      <x:c r="AI21" s="21"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="21"/>
@@ -1280,7 +1173,7 @@
       <x:c r="G22" s="21"/>
       <x:c r="H22" s="21"/>
       <x:c r="I22" s="21"/>
-      <x:c r="J22" s="28"/>
+      <x:c r="J22" s="21"/>
       <x:c r="K22" s="21"/>
       <x:c r="L22" s="21"/>
       <x:c r="M22" s="21"/>
@@ -1305,7 +1198,7 @@
       <x:c r="AF22" s="21"/>
       <x:c r="AG22" s="21"/>
       <x:c r="AH22" s="21"/>
-      <x:c r="AI22"/>
+      <x:c r="AI22" s="21"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="21"/>
@@ -1317,7 +1210,7 @@
       <x:c r="G23" s="21"/>
       <x:c r="H23" s="21"/>
       <x:c r="I23" s="21"/>
-      <x:c r="J23" s="28"/>
+      <x:c r="J23" s="21"/>
       <x:c r="K23" s="21"/>
       <x:c r="L23" s="21"/>
       <x:c r="M23" s="21"/>
@@ -1342,7 +1235,7 @@
       <x:c r="AF23" s="21"/>
       <x:c r="AG23" s="21"/>
       <x:c r="AH23" s="21"/>
-      <x:c r="AI23"/>
+      <x:c r="AI23" s="21"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="21"/>
@@ -1354,7 +1247,7 @@
       <x:c r="G24" s="21"/>
       <x:c r="H24" s="21"/>
       <x:c r="I24" s="21"/>
-      <x:c r="J24" s="28"/>
+      <x:c r="J24" s="21"/>
       <x:c r="K24" s="21"/>
       <x:c r="L24" s="21"/>
       <x:c r="M24" s="21"/>
@@ -1379,7 +1272,7 @@
       <x:c r="AF24" s="21"/>
       <x:c r="AG24" s="21"/>
       <x:c r="AH24" s="21"/>
-      <x:c r="AI24"/>
+      <x:c r="AI24" s="21"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="21"/>
@@ -1391,7 +1284,7 @@
       <x:c r="G25" s="21"/>
       <x:c r="H25" s="21"/>
       <x:c r="I25" s="21"/>
-      <x:c r="J25" s="28"/>
+      <x:c r="J25" s="21"/>
       <x:c r="K25" s="21"/>
       <x:c r="L25" s="21"/>
       <x:c r="M25" s="21"/>
@@ -1416,7 +1309,7 @@
       <x:c r="AF25" s="21"/>
       <x:c r="AG25" s="21"/>
       <x:c r="AH25" s="21"/>
-      <x:c r="AI25"/>
+      <x:c r="AI25" s="21"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="21"/>
@@ -1428,7 +1321,7 @@
       <x:c r="G26" s="21"/>
       <x:c r="H26" s="21"/>
       <x:c r="I26" s="21"/>
-      <x:c r="J26" s="28"/>
+      <x:c r="J26" s="21"/>
       <x:c r="K26" s="21"/>
       <x:c r="L26" s="21"/>
       <x:c r="M26" s="21"/>
@@ -1453,7 +1346,7 @@
       <x:c r="AF26" s="21"/>
       <x:c r="AG26" s="21"/>
       <x:c r="AH26" s="21"/>
-      <x:c r="AI26"/>
+      <x:c r="AI26" s="21"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="21"/>
@@ -1465,7 +1358,7 @@
       <x:c r="G27" s="21"/>
       <x:c r="H27" s="21"/>
       <x:c r="I27" s="21"/>
-      <x:c r="J27" s="28"/>
+      <x:c r="J27" s="21"/>
       <x:c r="K27" s="21"/>
       <x:c r="L27" s="21"/>
       <x:c r="M27" s="21"/>
@@ -1490,7 +1383,7 @@
       <x:c r="AF27" s="21"/>
       <x:c r="AG27" s="21"/>
       <x:c r="AH27" s="21"/>
-      <x:c r="AI27"/>
+      <x:c r="AI27" s="21"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="21"/>
@@ -1502,7 +1395,7 @@
       <x:c r="G28" s="21"/>
       <x:c r="H28" s="21"/>
       <x:c r="I28" s="21"/>
-      <x:c r="J28" s="28"/>
+      <x:c r="J28" s="21"/>
       <x:c r="K28" s="21"/>
       <x:c r="L28" s="21"/>
       <x:c r="M28" s="21"/>
@@ -1527,7 +1420,7 @@
       <x:c r="AF28" s="21"/>
       <x:c r="AG28" s="21"/>
       <x:c r="AH28" s="21"/>
-      <x:c r="AI28"/>
+      <x:c r="AI28" s="21"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="21"/>
@@ -1539,7 +1432,7 @@
       <x:c r="G29" s="21"/>
       <x:c r="H29" s="21"/>
       <x:c r="I29" s="21"/>
-      <x:c r="J29" s="28"/>
+      <x:c r="J29" s="21"/>
       <x:c r="K29" s="21"/>
       <x:c r="L29" s="21"/>
       <x:c r="M29" s="21"/>
@@ -1564,7 +1457,7 @@
       <x:c r="AF29" s="21"/>
       <x:c r="AG29" s="21"/>
       <x:c r="AH29" s="21"/>
-      <x:c r="AI29"/>
+      <x:c r="AI29" s="21"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="21"/>
@@ -1576,7 +1469,7 @@
       <x:c r="G30" s="21"/>
       <x:c r="H30" s="21"/>
       <x:c r="I30" s="21"/>
-      <x:c r="J30" s="28"/>
+      <x:c r="J30" s="21"/>
       <x:c r="K30" s="21"/>
       <x:c r="L30" s="21"/>
       <x:c r="M30" s="21"/>
@@ -1601,7 +1494,7 @@
       <x:c r="AF30" s="21"/>
       <x:c r="AG30" s="21"/>
       <x:c r="AH30" s="21"/>
-      <x:c r="AI30"/>
+      <x:c r="AI30" s="21"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="21"/>
@@ -1613,7 +1506,7 @@
       <x:c r="G31" s="21"/>
       <x:c r="H31" s="21"/>
       <x:c r="I31" s="21"/>
-      <x:c r="J31" s="28"/>
+      <x:c r="J31" s="21"/>
       <x:c r="K31" s="21"/>
       <x:c r="L31" s="21"/>
       <x:c r="M31" s="21"/>
@@ -1638,7 +1531,7 @@
       <x:c r="AF31" s="21"/>
       <x:c r="AG31" s="21"/>
       <x:c r="AH31" s="21"/>
-      <x:c r="AI31"/>
+      <x:c r="AI31" s="21"/>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="21"/>
@@ -1650,7 +1543,7 @@
       <x:c r="G32" s="21"/>
       <x:c r="H32" s="21"/>
       <x:c r="I32" s="21"/>
-      <x:c r="J32" s="28"/>
+      <x:c r="J32" s="21"/>
       <x:c r="K32" s="21"/>
       <x:c r="L32" s="21"/>
       <x:c r="M32" s="21"/>
@@ -1675,7 +1568,7 @@
       <x:c r="AF32" s="21"/>
       <x:c r="AG32" s="21"/>
       <x:c r="AH32" s="21"/>
-      <x:c r="AI32"/>
+      <x:c r="AI32" s="21"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="21"/>
@@ -1687,7 +1580,7 @@
       <x:c r="G33" s="21"/>
       <x:c r="H33" s="21"/>
       <x:c r="I33" s="21"/>
-      <x:c r="J33" s="28"/>
+      <x:c r="J33" s="21"/>
       <x:c r="K33" s="21"/>
       <x:c r="L33" s="21"/>
       <x:c r="M33" s="21"/>
@@ -1712,7 +1605,7 @@
       <x:c r="AF33" s="21"/>
       <x:c r="AG33" s="21"/>
       <x:c r="AH33" s="21"/>
-      <x:c r="AI33"/>
+      <x:c r="AI33" s="21"/>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="21"/>
@@ -1724,7 +1617,7 @@
       <x:c r="G34" s="21"/>
       <x:c r="H34" s="21"/>
       <x:c r="I34" s="21"/>
-      <x:c r="J34" s="28"/>
+      <x:c r="J34" s="21"/>
       <x:c r="K34" s="21"/>
       <x:c r="L34" s="21"/>
       <x:c r="M34" s="21"/>
@@ -1749,7 +1642,7 @@
       <x:c r="AF34" s="21"/>
       <x:c r="AG34" s="21"/>
       <x:c r="AH34" s="21"/>
-      <x:c r="AI34"/>
+      <x:c r="AI34" s="21"/>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="21"/>
@@ -1761,7 +1654,7 @@
       <x:c r="G35" s="21"/>
       <x:c r="H35" s="21"/>
       <x:c r="I35" s="21"/>
-      <x:c r="J35" s="28"/>
+      <x:c r="J35" s="21"/>
       <x:c r="K35" s="21"/>
       <x:c r="L35" s="21"/>
       <x:c r="M35" s="21"/>
@@ -1786,7 +1679,7 @@
       <x:c r="AF35" s="21"/>
       <x:c r="AG35" s="21"/>
       <x:c r="AH35" s="21"/>
-      <x:c r="AI35"/>
+      <x:c r="AI35" s="21"/>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="21"/>
@@ -1798,7 +1691,7 @@
       <x:c r="G36" s="21"/>
       <x:c r="H36" s="21"/>
       <x:c r="I36" s="21"/>
-      <x:c r="J36" s="28"/>
+      <x:c r="J36" s="21"/>
       <x:c r="K36" s="21"/>
       <x:c r="L36" s="21"/>
       <x:c r="M36" s="21"/>
@@ -1823,7 +1716,7 @@
       <x:c r="AF36" s="21"/>
       <x:c r="AG36" s="21"/>
       <x:c r="AH36" s="21"/>
-      <x:c r="AI36"/>
+      <x:c r="AI36" s="21"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="21"/>
@@ -1835,7 +1728,7 @@
       <x:c r="G37" s="21"/>
       <x:c r="H37" s="21"/>
       <x:c r="I37" s="21"/>
-      <x:c r="J37" s="28"/>
+      <x:c r="J37" s="21"/>
       <x:c r="K37" s="21"/>
       <x:c r="L37" s="21"/>
       <x:c r="M37" s="21"/>
@@ -1860,7 +1753,7 @@
       <x:c r="AF37" s="21"/>
       <x:c r="AG37" s="21"/>
       <x:c r="AH37" s="21"/>
-      <x:c r="AI37"/>
+      <x:c r="AI37" s="21"/>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="21"/>
@@ -1872,7 +1765,7 @@
       <x:c r="G38" s="21"/>
       <x:c r="H38" s="21"/>
       <x:c r="I38" s="21"/>
-      <x:c r="J38" s="28"/>
+      <x:c r="J38" s="21"/>
       <x:c r="K38" s="21"/>
       <x:c r="L38" s="21"/>
       <x:c r="M38" s="21"/>
@@ -1897,7 +1790,7 @@
       <x:c r="AF38" s="21"/>
       <x:c r="AG38" s="21"/>
       <x:c r="AH38" s="21"/>
-      <x:c r="AI38"/>
+      <x:c r="AI38" s="21"/>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="21"/>
@@ -1909,7 +1802,7 @@
       <x:c r="G39" s="21"/>
       <x:c r="H39" s="21"/>
       <x:c r="I39" s="21"/>
-      <x:c r="J39" s="28"/>
+      <x:c r="J39" s="21"/>
       <x:c r="K39" s="21"/>
       <x:c r="L39" s="21"/>
       <x:c r="M39" s="21"/>
@@ -1934,7 +1827,7 @@
       <x:c r="AF39" s="21"/>
       <x:c r="AG39" s="21"/>
       <x:c r="AH39" s="21"/>
-      <x:c r="AI39"/>
+      <x:c r="AI39" s="21"/>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="21"/>
@@ -1946,7 +1839,7 @@
       <x:c r="G40" s="21"/>
       <x:c r="H40" s="21"/>
       <x:c r="I40" s="21"/>
-      <x:c r="J40" s="28"/>
+      <x:c r="J40" s="21"/>
       <x:c r="K40" s="21"/>
       <x:c r="L40" s="21"/>
       <x:c r="M40" s="21"/>
@@ -1971,7 +1864,7 @@
       <x:c r="AF40" s="21"/>
       <x:c r="AG40" s="21"/>
       <x:c r="AH40" s="21"/>
-      <x:c r="AI40"/>
+      <x:c r="AI40" s="21"/>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="21"/>
@@ -1983,7 +1876,7 @@
       <x:c r="G41" s="21"/>
       <x:c r="H41" s="21"/>
       <x:c r="I41" s="21"/>
-      <x:c r="J41" s="28"/>
+      <x:c r="J41" s="21"/>
       <x:c r="K41" s="21"/>
       <x:c r="L41" s="21"/>
       <x:c r="M41" s="21"/>
@@ -2008,7 +1901,7 @@
       <x:c r="AF41" s="21"/>
       <x:c r="AG41" s="21"/>
       <x:c r="AH41" s="21"/>
-      <x:c r="AI41"/>
+      <x:c r="AI41" s="21"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="21"/>
@@ -2020,7 +1913,7 @@
       <x:c r="G42" s="21"/>
       <x:c r="H42" s="21"/>
       <x:c r="I42" s="21"/>
-      <x:c r="J42" s="28"/>
+      <x:c r="J42" s="21"/>
       <x:c r="K42" s="21"/>
       <x:c r="L42" s="21"/>
       <x:c r="M42" s="21"/>
@@ -2045,7 +1938,7 @@
       <x:c r="AF42" s="21"/>
       <x:c r="AG42" s="21"/>
       <x:c r="AH42" s="21"/>
-      <x:c r="AI42"/>
+      <x:c r="AI42" s="21"/>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="21"/>
@@ -2057,7 +1950,7 @@
       <x:c r="G43" s="21"/>
       <x:c r="H43" s="21"/>
       <x:c r="I43" s="21"/>
-      <x:c r="J43" s="28"/>
+      <x:c r="J43" s="21"/>
       <x:c r="K43" s="21"/>
       <x:c r="L43" s="21"/>
       <x:c r="M43" s="21"/>
@@ -2082,7 +1975,7 @@
       <x:c r="AF43" s="21"/>
       <x:c r="AG43" s="21"/>
       <x:c r="AH43" s="21"/>
-      <x:c r="AI43"/>
+      <x:c r="AI43" s="21"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="21"/>
@@ -2094,7 +1987,7 @@
       <x:c r="G44" s="21"/>
       <x:c r="H44" s="21"/>
       <x:c r="I44" s="21"/>
-      <x:c r="J44" s="28"/>
+      <x:c r="J44" s="21"/>
       <x:c r="K44" s="21"/>
       <x:c r="L44" s="21"/>
       <x:c r="M44" s="21"/>
@@ -2119,7 +2012,7 @@
       <x:c r="AF44" s="21"/>
       <x:c r="AG44" s="21"/>
       <x:c r="AH44" s="21"/>
-      <x:c r="AI44"/>
+      <x:c r="AI44" s="21"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="21"/>
@@ -2131,7 +2024,7 @@
       <x:c r="G45" s="21"/>
       <x:c r="H45" s="21"/>
       <x:c r="I45" s="21"/>
-      <x:c r="J45" s="28"/>
+      <x:c r="J45" s="21"/>
       <x:c r="K45" s="21"/>
       <x:c r="L45" s="21"/>
       <x:c r="M45" s="21"/>
@@ -2156,7 +2049,7 @@
       <x:c r="AF45" s="21"/>
       <x:c r="AG45" s="21"/>
       <x:c r="AH45" s="21"/>
-      <x:c r="AI45"/>
+      <x:c r="AI45" s="21"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="21"/>
@@ -2168,7 +2061,7 @@
       <x:c r="G46" s="21"/>
       <x:c r="H46" s="21"/>
       <x:c r="I46" s="21"/>
-      <x:c r="J46" s="28"/>
+      <x:c r="J46" s="21"/>
       <x:c r="K46" s="21"/>
       <x:c r="L46" s="21"/>
       <x:c r="M46" s="21"/>
@@ -2193,7 +2086,7 @@
       <x:c r="AF46" s="21"/>
       <x:c r="AG46" s="21"/>
       <x:c r="AH46" s="21"/>
-      <x:c r="AI46"/>
+      <x:c r="AI46" s="21"/>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="21"/>
@@ -2205,7 +2098,7 @@
       <x:c r="G47" s="21"/>
       <x:c r="H47" s="21"/>
       <x:c r="I47" s="21"/>
-      <x:c r="J47" s="28"/>
+      <x:c r="J47" s="21"/>
       <x:c r="K47" s="21"/>
       <x:c r="L47" s="21"/>
       <x:c r="M47" s="21"/>
@@ -2230,7 +2123,7 @@
       <x:c r="AF47" s="21"/>
       <x:c r="AG47" s="21"/>
       <x:c r="AH47" s="21"/>
-      <x:c r="AI47"/>
+      <x:c r="AI47" s="21"/>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="21"/>
@@ -2242,7 +2135,7 @@
       <x:c r="G48" s="21"/>
       <x:c r="H48" s="21"/>
       <x:c r="I48" s="21"/>
-      <x:c r="J48" s="28"/>
+      <x:c r="J48" s="21"/>
       <x:c r="K48" s="21"/>
       <x:c r="L48" s="21"/>
       <x:c r="M48" s="21"/>
@@ -2267,7 +2160,7 @@
       <x:c r="AF48" s="21"/>
       <x:c r="AG48" s="21"/>
       <x:c r="AH48" s="21"/>
-      <x:c r="AI48"/>
+      <x:c r="AI48" s="21"/>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="21"/>
@@ -2279,7 +2172,7 @@
       <x:c r="G49" s="21"/>
       <x:c r="H49" s="21"/>
       <x:c r="I49" s="21"/>
-      <x:c r="J49" s="28"/>
+      <x:c r="J49" s="21"/>
       <x:c r="K49" s="21"/>
       <x:c r="L49" s="21"/>
       <x:c r="M49" s="21"/>
@@ -2304,7 +2197,7 @@
       <x:c r="AF49" s="21"/>
       <x:c r="AG49" s="21"/>
       <x:c r="AH49" s="21"/>
-      <x:c r="AI49"/>
+      <x:c r="AI49" s="21"/>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="21"/>
@@ -2316,7 +2209,7 @@
       <x:c r="G50" s="21"/>
       <x:c r="H50" s="21"/>
       <x:c r="I50" s="21"/>
-      <x:c r="J50" s="28"/>
+      <x:c r="J50" s="21"/>
       <x:c r="K50" s="21"/>
       <x:c r="L50" s="21"/>
       <x:c r="M50" s="21"/>
@@ -2341,7 +2234,7 @@
       <x:c r="AF50" s="21"/>
       <x:c r="AG50" s="21"/>
       <x:c r="AH50" s="21"/>
-      <x:c r="AI50"/>
+      <x:c r="AI50" s="21"/>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="21"/>
@@ -2353,7 +2246,7 @@
       <x:c r="G51" s="21"/>
       <x:c r="H51" s="21"/>
       <x:c r="I51" s="21"/>
-      <x:c r="J51" s="28"/>
+      <x:c r="J51" s="21"/>
       <x:c r="K51" s="21"/>
       <x:c r="L51" s="21"/>
       <x:c r="M51" s="21"/>
@@ -2378,7 +2271,7 @@
       <x:c r="AF51" s="21"/>
       <x:c r="AG51" s="21"/>
       <x:c r="AH51" s="21"/>
-      <x:c r="AI51"/>
+      <x:c r="AI51" s="21"/>
     </x:row>
     <x:row r="52" ht="23" customHeight="1">
       <x:c r="A52" s="21"/>
@@ -2390,7 +2283,7 @@
       <x:c r="G52" s="21"/>
       <x:c r="H52" s="21"/>
       <x:c r="I52" s="21"/>
-      <x:c r="J52" s="28"/>
+      <x:c r="J52" s="21"/>
       <x:c r="K52" s="21"/>
       <x:c r="L52" s="21"/>
       <x:c r="M52" s="21"/>
@@ -2415,7 +2308,7 @@
       <x:c r="AF52" s="21"/>
       <x:c r="AG52" s="21"/>
       <x:c r="AH52" s="21"/>
-      <x:c r="AI52"/>
+      <x:c r="AI52" s="21"/>
     </x:row>
     <x:row r="53" ht="23" customHeight="1">
       <x:c r="A53" s="21"/>
@@ -2427,7 +2320,7 @@
       <x:c r="G53" s="21"/>
       <x:c r="H53" s="21"/>
       <x:c r="I53" s="21"/>
-      <x:c r="J53" s="28"/>
+      <x:c r="J53" s="21"/>
       <x:c r="K53" s="21"/>
       <x:c r="L53" s="21"/>
       <x:c r="M53" s="21"/>
@@ -2452,7 +2345,7 @@
       <x:c r="AF53" s="21"/>
       <x:c r="AG53" s="21"/>
       <x:c r="AH53" s="21"/>
-      <x:c r="AI53"/>
+      <x:c r="AI53" s="21"/>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
       <x:c r="A54" s="21"/>
@@ -2464,7 +2357,7 @@
       <x:c r="G54" s="21"/>
       <x:c r="H54" s="21"/>
       <x:c r="I54" s="21"/>
-      <x:c r="J54" s="28"/>
+      <x:c r="J54" s="21"/>
       <x:c r="K54" s="21"/>
       <x:c r="L54" s="21"/>
       <x:c r="M54" s="21"/>
@@ -2489,7 +2382,7 @@
       <x:c r="AF54" s="21"/>
       <x:c r="AG54" s="21"/>
       <x:c r="AH54" s="21"/>
-      <x:c r="AI54"/>
+      <x:c r="AI54" s="21"/>
     </x:row>
     <x:row r="55" ht="23" customHeight="1">
       <x:c r="A55" s="21"/>
@@ -2501,7 +2394,7 @@
       <x:c r="G55" s="21"/>
       <x:c r="H55" s="21"/>
       <x:c r="I55" s="21"/>
-      <x:c r="J55" s="28"/>
+      <x:c r="J55" s="21"/>
       <x:c r="K55" s="21"/>
       <x:c r="L55" s="21"/>
       <x:c r="M55" s="21"/>
@@ -2526,7 +2419,7 @@
       <x:c r="AF55" s="21"/>
       <x:c r="AG55" s="21"/>
       <x:c r="AH55" s="21"/>
-      <x:c r="AI55"/>
+      <x:c r="AI55" s="21"/>
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
       <x:c r="A56" s="21"/>
@@ -2538,7 +2431,7 @@
       <x:c r="G56" s="21"/>
       <x:c r="H56" s="21"/>
       <x:c r="I56" s="21"/>
-      <x:c r="J56" s="28"/>
+      <x:c r="J56" s="21"/>
       <x:c r="K56" s="21"/>
       <x:c r="L56" s="21"/>
       <x:c r="M56" s="21"/>
@@ -2563,7 +2456,7 @@
       <x:c r="AF56" s="21"/>
       <x:c r="AG56" s="21"/>
       <x:c r="AH56" s="21"/>
-      <x:c r="AI56"/>
+      <x:c r="AI56" s="21"/>
     </x:row>
     <x:row r="57" ht="23" customHeight="1">
       <x:c r="A57" s="21"/>
@@ -2575,7 +2468,7 @@
       <x:c r="G57" s="21"/>
       <x:c r="H57" s="21"/>
       <x:c r="I57" s="21"/>
-      <x:c r="J57" s="28"/>
+      <x:c r="J57" s="21"/>
       <x:c r="K57" s="21"/>
       <x:c r="L57" s="21"/>
       <x:c r="M57" s="21"/>
@@ -2600,7 +2493,7 @@
       <x:c r="AF57" s="21"/>
       <x:c r="AG57" s="21"/>
       <x:c r="AH57" s="21"/>
-      <x:c r="AI57"/>
+      <x:c r="AI57" s="21"/>
     </x:row>
     <x:row r="58" ht="23" customHeight="1">
       <x:c r="A58" s="21"/>
@@ -2612,7 +2505,7 @@
       <x:c r="G58" s="21"/>
       <x:c r="H58" s="21"/>
       <x:c r="I58" s="21"/>
-      <x:c r="J58" s="28"/>
+      <x:c r="J58" s="21"/>
       <x:c r="K58" s="21"/>
       <x:c r="L58" s="21"/>
       <x:c r="M58" s="21"/>
@@ -2637,7 +2530,7 @@
       <x:c r="AF58" s="21"/>
       <x:c r="AG58" s="21"/>
       <x:c r="AH58" s="21"/>
-      <x:c r="AI58"/>
+      <x:c r="AI58" s="21"/>
     </x:row>
     <x:row r="59" ht="23" customHeight="1">
       <x:c r="A59" s="21"/>
@@ -2649,7 +2542,7 @@
       <x:c r="G59" s="21"/>
       <x:c r="H59" s="21"/>
       <x:c r="I59" s="21"/>
-      <x:c r="J59" s="28"/>
+      <x:c r="J59" s="21"/>
       <x:c r="K59" s="21"/>
       <x:c r="L59" s="21"/>
       <x:c r="M59" s="21"/>
@@ -2674,7 +2567,7 @@
       <x:c r="AF59" s="21"/>
       <x:c r="AG59" s="21"/>
       <x:c r="AH59" s="21"/>
-      <x:c r="AI59"/>
+      <x:c r="AI59" s="21"/>
     </x:row>
     <x:row r="60" ht="23" customHeight="1">
       <x:c r="A60" s="21"/>
@@ -2686,7 +2579,7 @@
       <x:c r="G60" s="21"/>
       <x:c r="H60" s="21"/>
       <x:c r="I60" s="21"/>
-      <x:c r="J60" s="28"/>
+      <x:c r="J60" s="21"/>
       <x:c r="K60" s="21"/>
       <x:c r="L60" s="21"/>
       <x:c r="M60" s="21"/>
@@ -2711,7 +2604,7 @@
       <x:c r="AF60" s="21"/>
       <x:c r="AG60" s="21"/>
       <x:c r="AH60" s="21"/>
-      <x:c r="AI60"/>
+      <x:c r="AI60" s="21"/>
     </x:row>
     <x:row r="61" ht="23" customHeight="1">
       <x:c r="A61" s="21"/>
@@ -2723,7 +2616,7 @@
       <x:c r="G61" s="21"/>
       <x:c r="H61" s="21"/>
       <x:c r="I61" s="21"/>
-      <x:c r="J61" s="28"/>
+      <x:c r="J61" s="21"/>
       <x:c r="K61" s="21"/>
       <x:c r="L61" s="21"/>
       <x:c r="M61" s="21"/>
@@ -2748,7 +2641,7 @@
       <x:c r="AF61" s="21"/>
       <x:c r="AG61" s="21"/>
       <x:c r="AH61" s="21"/>
-      <x:c r="AI61"/>
+      <x:c r="AI61" s="21"/>
     </x:row>
     <x:row r="62" ht="23" customHeight="1">
       <x:c r="A62" s="21"/>
@@ -2760,7 +2653,7 @@
       <x:c r="G62" s="21"/>
       <x:c r="H62" s="21"/>
       <x:c r="I62" s="21"/>
-      <x:c r="J62" s="28"/>
+      <x:c r="J62" s="21"/>
       <x:c r="K62" s="21"/>
       <x:c r="L62" s="21"/>
       <x:c r="M62" s="21"/>
@@ -2785,7 +2678,7 @@
       <x:c r="AF62" s="21"/>
       <x:c r="AG62" s="21"/>
       <x:c r="AH62" s="21"/>
-      <x:c r="AI62"/>
+      <x:c r="AI62" s="21"/>
     </x:row>
     <x:row r="63" ht="23" customHeight="1">
       <x:c r="A63" s="21"/>
@@ -2797,7 +2690,7 @@
       <x:c r="G63" s="21"/>
       <x:c r="H63" s="21"/>
       <x:c r="I63" s="21"/>
-      <x:c r="J63" s="28"/>
+      <x:c r="J63" s="21"/>
       <x:c r="K63" s="21"/>
       <x:c r="L63" s="21"/>
       <x:c r="M63" s="21"/>
@@ -2822,7 +2715,7 @@
       <x:c r="AF63" s="21"/>
       <x:c r="AG63" s="21"/>
       <x:c r="AH63" s="21"/>
-      <x:c r="AI63"/>
+      <x:c r="AI63" s="21"/>
     </x:row>
     <x:row r="64" ht="23" customHeight="1">
       <x:c r="A64" s="21"/>
@@ -2834,7 +2727,7 @@
       <x:c r="G64" s="21"/>
       <x:c r="H64" s="21"/>
       <x:c r="I64" s="21"/>
-      <x:c r="J64" s="28"/>
+      <x:c r="J64" s="21"/>
       <x:c r="K64" s="21"/>
       <x:c r="L64" s="21"/>
       <x:c r="M64" s="21"/>
@@ -2859,7 +2752,7 @@
       <x:c r="AF64" s="21"/>
       <x:c r="AG64" s="21"/>
       <x:c r="AH64" s="21"/>
-      <x:c r="AI64"/>
+      <x:c r="AI64" s="21"/>
     </x:row>
     <x:row r="65" ht="23" customHeight="1">
       <x:c r="A65" s="21"/>
@@ -2871,7 +2764,7 @@
       <x:c r="G65" s="21"/>
       <x:c r="H65" s="21"/>
       <x:c r="I65" s="21"/>
-      <x:c r="J65" s="28"/>
+      <x:c r="J65" s="21"/>
       <x:c r="K65" s="21"/>
       <x:c r="L65" s="21"/>
       <x:c r="M65" s="21"/>
@@ -2896,7 +2789,7 @@
       <x:c r="AF65" s="21"/>
       <x:c r="AG65" s="21"/>
       <x:c r="AH65" s="21"/>
-      <x:c r="AI65"/>
+      <x:c r="AI65" s="21"/>
     </x:row>
     <x:row r="66" ht="23" customHeight="1">
       <x:c r="A66" s="21"/>
@@ -2908,7 +2801,7 @@
       <x:c r="G66" s="21"/>
       <x:c r="H66" s="21"/>
       <x:c r="I66" s="21"/>
-      <x:c r="J66" s="28"/>
+      <x:c r="J66" s="21"/>
       <x:c r="K66" s="21"/>
       <x:c r="L66" s="21"/>
       <x:c r="M66" s="21"/>
@@ -2933,7 +2826,7 @@
       <x:c r="AF66" s="21"/>
       <x:c r="AG66" s="21"/>
       <x:c r="AH66" s="21"/>
-      <x:c r="AI66"/>
+      <x:c r="AI66" s="21"/>
     </x:row>
     <x:row r="67" ht="23" customHeight="1">
       <x:c r="A67" s="21"/>
@@ -2945,7 +2838,7 @@
       <x:c r="G67" s="21"/>
       <x:c r="H67" s="21"/>
       <x:c r="I67" s="21"/>
-      <x:c r="J67" s="28"/>
+      <x:c r="J67" s="21"/>
       <x:c r="K67" s="21"/>
       <x:c r="L67" s="21"/>
       <x:c r="M67" s="21"/>
@@ -2970,7 +2863,7 @@
       <x:c r="AF67" s="21"/>
       <x:c r="AG67" s="21"/>
       <x:c r="AH67" s="21"/>
-      <x:c r="AI67"/>
+      <x:c r="AI67" s="21"/>
     </x:row>
     <x:row r="68" ht="23" customHeight="1">
       <x:c r="A68" s="21"/>
@@ -2982,7 +2875,7 @@
       <x:c r="G68" s="21"/>
       <x:c r="H68" s="21"/>
       <x:c r="I68" s="21"/>
-      <x:c r="J68" s="28"/>
+      <x:c r="J68" s="21"/>
       <x:c r="K68" s="21"/>
       <x:c r="L68" s="21"/>
       <x:c r="M68" s="21"/>
@@ -3007,7 +2900,7 @@
       <x:c r="AF68" s="21"/>
       <x:c r="AG68" s="21"/>
       <x:c r="AH68" s="21"/>
-      <x:c r="AI68"/>
+      <x:c r="AI68" s="21"/>
     </x:row>
     <x:row r="69" ht="23" customHeight="1">
       <x:c r="A69" s="21"/>
@@ -3019,7 +2912,7 @@
       <x:c r="G69" s="21"/>
       <x:c r="H69" s="21"/>
       <x:c r="I69" s="21"/>
-      <x:c r="J69" s="28"/>
+      <x:c r="J69" s="21"/>
       <x:c r="K69" s="21"/>
       <x:c r="L69" s="21"/>
       <x:c r="M69" s="21"/>
@@ -3044,7 +2937,7 @@
       <x:c r="AF69" s="21"/>
       <x:c r="AG69" s="21"/>
       <x:c r="AH69" s="21"/>
-      <x:c r="AI69"/>
+      <x:c r="AI69" s="21"/>
     </x:row>
     <x:row r="70" ht="23" customHeight="1">
       <x:c r="A70" s="21"/>
@@ -3056,7 +2949,7 @@
       <x:c r="G70" s="21"/>
       <x:c r="H70" s="21"/>
       <x:c r="I70" s="21"/>
-      <x:c r="J70" s="28"/>
+      <x:c r="J70" s="21"/>
       <x:c r="K70" s="21"/>
       <x:c r="L70" s="21"/>
       <x:c r="M70" s="21"/>
@@ -3081,7 +2974,7 @@
       <x:c r="AF70" s="21"/>
       <x:c r="AG70" s="21"/>
       <x:c r="AH70" s="21"/>
-      <x:c r="AI70"/>
+      <x:c r="AI70" s="21"/>
     </x:row>
     <x:row r="71" ht="23" customHeight="1">
       <x:c r="A71" s="21"/>
@@ -3093,7 +2986,7 @@
       <x:c r="G71" s="21"/>
       <x:c r="H71" s="21"/>
       <x:c r="I71" s="21"/>
-      <x:c r="J71" s="28"/>
+      <x:c r="J71" s="21"/>
       <x:c r="K71" s="21"/>
       <x:c r="L71" s="21"/>
       <x:c r="M71" s="21"/>
@@ -3118,7 +3011,7 @@
       <x:c r="AF71" s="21"/>
       <x:c r="AG71" s="21"/>
       <x:c r="AH71" s="21"/>
-      <x:c r="AI71"/>
+      <x:c r="AI71" s="21"/>
     </x:row>
     <x:row r="72" ht="23" customHeight="1">
       <x:c r="A72" s="21"/>
@@ -3130,7 +3023,7 @@
       <x:c r="G72" s="21"/>
       <x:c r="H72" s="21"/>
       <x:c r="I72" s="21"/>
-      <x:c r="J72" s="28"/>
+      <x:c r="J72" s="21"/>
       <x:c r="K72" s="21"/>
       <x:c r="L72" s="21"/>
       <x:c r="M72" s="21"/>
@@ -3155,7 +3048,7 @@
       <x:c r="AF72" s="21"/>
       <x:c r="AG72" s="21"/>
       <x:c r="AH72" s="21"/>
-      <x:c r="AI72"/>
+      <x:c r="AI72" s="21"/>
     </x:row>
     <x:row r="73" ht="23" customHeight="1">
       <x:c r="A73" s="21"/>
@@ -3167,7 +3060,7 @@
       <x:c r="G73" s="21"/>
       <x:c r="H73" s="21"/>
       <x:c r="I73" s="21"/>
-      <x:c r="J73" s="28"/>
+      <x:c r="J73" s="21"/>
       <x:c r="K73" s="21"/>
       <x:c r="L73" s="21"/>
       <x:c r="M73" s="21"/>
@@ -3192,7 +3085,7 @@
       <x:c r="AF73" s="21"/>
       <x:c r="AG73" s="21"/>
       <x:c r="AH73" s="21"/>
-      <x:c r="AI73"/>
+      <x:c r="AI73" s="21"/>
     </x:row>
     <x:row r="74" ht="23" customHeight="1">
       <x:c r="A74" s="21"/>
@@ -3204,7 +3097,7 @@
       <x:c r="G74" s="21"/>
       <x:c r="H74" s="21"/>
       <x:c r="I74" s="21"/>
-      <x:c r="J74" s="28"/>
+      <x:c r="J74" s="21"/>
       <x:c r="K74" s="21"/>
       <x:c r="L74" s="21"/>
       <x:c r="M74" s="21"/>
@@ -3229,7 +3122,7 @@
       <x:c r="AF74" s="21"/>
       <x:c r="AG74" s="21"/>
       <x:c r="AH74" s="21"/>
-      <x:c r="AI74"/>
+      <x:c r="AI74" s="21"/>
     </x:row>
     <x:row r="75" ht="23" customHeight="1">
       <x:c r="A75" s="21"/>
@@ -3241,7 +3134,7 @@
       <x:c r="G75" s="21"/>
       <x:c r="H75" s="21"/>
       <x:c r="I75" s="21"/>
-      <x:c r="J75" s="28"/>
+      <x:c r="J75" s="21"/>
       <x:c r="K75" s="21"/>
       <x:c r="L75" s="21"/>
       <x:c r="M75" s="21"/>
@@ -3266,7 +3159,7 @@
       <x:c r="AF75" s="21"/>
       <x:c r="AG75" s="21"/>
       <x:c r="AH75" s="21"/>
-      <x:c r="AI75"/>
+      <x:c r="AI75" s="21"/>
     </x:row>
     <x:row r="76" ht="23" customHeight="1">
       <x:c r="A76" s="21"/>
@@ -3278,7 +3171,7 @@
       <x:c r="G76" s="21"/>
       <x:c r="H76" s="21"/>
       <x:c r="I76" s="21"/>
-      <x:c r="J76" s="28"/>
+      <x:c r="J76" s="21"/>
       <x:c r="K76" s="21"/>
       <x:c r="L76" s="21"/>
       <x:c r="M76" s="21"/>
@@ -3303,7 +3196,7 @@
       <x:c r="AF76" s="21"/>
       <x:c r="AG76" s="21"/>
       <x:c r="AH76" s="21"/>
-      <x:c r="AI76"/>
+      <x:c r="AI76" s="21"/>
     </x:row>
     <x:row r="77" ht="23" customHeight="1">
       <x:c r="A77" s="21"/>
@@ -3315,7 +3208,7 @@
       <x:c r="G77" s="21"/>
       <x:c r="H77" s="21"/>
       <x:c r="I77" s="21"/>
-      <x:c r="J77" s="28"/>
+      <x:c r="J77" s="21"/>
       <x:c r="K77" s="21"/>
       <x:c r="L77" s="21"/>
       <x:c r="M77" s="21"/>
@@ -3340,7 +3233,7 @@
       <x:c r="AF77" s="21"/>
       <x:c r="AG77" s="21"/>
       <x:c r="AH77" s="21"/>
-      <x:c r="AI77"/>
+      <x:c r="AI77" s="21"/>
     </x:row>
     <x:row r="78" ht="23" customHeight="1">
       <x:c r="A78" s="21"/>
@@ -3352,7 +3245,7 @@
       <x:c r="G78" s="21"/>
       <x:c r="H78" s="21"/>
       <x:c r="I78" s="21"/>
-      <x:c r="J78" s="28"/>
+      <x:c r="J78" s="21"/>
       <x:c r="K78" s="21"/>
       <x:c r="L78" s="21"/>
       <x:c r="M78" s="21"/>
@@ -3377,7 +3270,7 @@
       <x:c r="AF78" s="21"/>
       <x:c r="AG78" s="21"/>
       <x:c r="AH78" s="21"/>
-      <x:c r="AI78"/>
+      <x:c r="AI78" s="21"/>
     </x:row>
     <x:row r="79" ht="23" customHeight="1">
       <x:c r="A79" s="21"/>
@@ -3389,7 +3282,7 @@
       <x:c r="G79" s="21"/>
       <x:c r="H79" s="21"/>
       <x:c r="I79" s="21"/>
-      <x:c r="J79" s="28"/>
+      <x:c r="J79" s="21"/>
       <x:c r="K79" s="21"/>
       <x:c r="L79" s="21"/>
       <x:c r="M79" s="21"/>
@@ -3414,7 +3307,7 @@
       <x:c r="AF79" s="21"/>
       <x:c r="AG79" s="21"/>
       <x:c r="AH79" s="21"/>
-      <x:c r="AI79"/>
+      <x:c r="AI79" s="21"/>
     </x:row>
     <x:row r="80" ht="23" customHeight="1">
       <x:c r="A80" s="21"/>
@@ -3426,7 +3319,7 @@
       <x:c r="G80" s="21"/>
       <x:c r="H80" s="21"/>
       <x:c r="I80" s="21"/>
-      <x:c r="J80" s="28"/>
+      <x:c r="J80" s="21"/>
       <x:c r="K80" s="21"/>
       <x:c r="L80" s="21"/>
       <x:c r="M80" s="21"/>
@@ -3451,7 +3344,7 @@
       <x:c r="AF80" s="21"/>
       <x:c r="AG80" s="21"/>
       <x:c r="AH80" s="21"/>
-      <x:c r="AI80"/>
+      <x:c r="AI80" s="21"/>
     </x:row>
     <x:row r="81" ht="23" customHeight="1">
       <x:c r="A81" s="21"/>
@@ -3463,7 +3356,7 @@
       <x:c r="G81" s="21"/>
       <x:c r="H81" s="21"/>
       <x:c r="I81" s="21"/>
-      <x:c r="J81" s="28"/>
+      <x:c r="J81" s="21"/>
       <x:c r="K81" s="21"/>
       <x:c r="L81" s="21"/>
       <x:c r="M81" s="21"/>
@@ -3488,7 +3381,7 @@
       <x:c r="AF81" s="21"/>
       <x:c r="AG81" s="21"/>
       <x:c r="AH81" s="21"/>
-      <x:c r="AI81"/>
+      <x:c r="AI81" s="21"/>
     </x:row>
     <x:row r="82" ht="23" customHeight="1">
       <x:c r="A82" s="21"/>
@@ -3500,7 +3393,7 @@
       <x:c r="G82" s="21"/>
       <x:c r="H82" s="21"/>
       <x:c r="I82" s="21"/>
-      <x:c r="J82" s="28"/>
+      <x:c r="J82" s="21"/>
       <x:c r="K82" s="21"/>
       <x:c r="L82" s="21"/>
       <x:c r="M82" s="21"/>
@@ -3525,7 +3418,7 @@
       <x:c r="AF82" s="21"/>
       <x:c r="AG82" s="21"/>
       <x:c r="AH82" s="21"/>
-      <x:c r="AI82"/>
+      <x:c r="AI82" s="21"/>
     </x:row>
     <x:row r="83" ht="23" customHeight="1">
       <x:c r="A83" s="21"/>
@@ -3537,7 +3430,7 @@
       <x:c r="G83" s="21"/>
       <x:c r="H83" s="21"/>
       <x:c r="I83" s="21"/>
-      <x:c r="J83" s="28"/>
+      <x:c r="J83" s="21"/>
       <x:c r="K83" s="21"/>
       <x:c r="L83" s="21"/>
       <x:c r="M83" s="21"/>
@@ -3562,7 +3455,7 @@
       <x:c r="AF83" s="21"/>
       <x:c r="AG83" s="21"/>
       <x:c r="AH83" s="21"/>
-      <x:c r="AI83"/>
+      <x:c r="AI83" s="21"/>
     </x:row>
     <x:row r="84" ht="23" customHeight="1">
       <x:c r="A84" s="21"/>
@@ -3574,7 +3467,7 @@
       <x:c r="G84" s="21"/>
       <x:c r="H84" s="21"/>
       <x:c r="I84" s="21"/>
-      <x:c r="J84" s="28"/>
+      <x:c r="J84" s="21"/>
       <x:c r="K84" s="21"/>
       <x:c r="L84" s="21"/>
       <x:c r="M84" s="21"/>
@@ -3599,7 +3492,7 @@
       <x:c r="AF84" s="21"/>
       <x:c r="AG84" s="21"/>
       <x:c r="AH84" s="21"/>
-      <x:c r="AI84"/>
+      <x:c r="AI84" s="21"/>
     </x:row>
     <x:row r="85" ht="23" customHeight="1">
       <x:c r="A85" s="21"/>
@@ -3611,7 +3504,7 @@
       <x:c r="G85" s="21"/>
       <x:c r="H85" s="21"/>
       <x:c r="I85" s="21"/>
-      <x:c r="J85" s="28"/>
+      <x:c r="J85" s="21"/>
       <x:c r="K85" s="21"/>
       <x:c r="L85" s="21"/>
       <x:c r="M85" s="21"/>
@@ -3636,7 +3529,7 @@
       <x:c r="AF85" s="21"/>
       <x:c r="AG85" s="21"/>
       <x:c r="AH85" s="21"/>
-      <x:c r="AI85"/>
+      <x:c r="AI85" s="21"/>
     </x:row>
     <x:row r="86" ht="23" customHeight="1">
       <x:c r="A86" s="21"/>
@@ -3648,7 +3541,7 @@
       <x:c r="G86" s="21"/>
       <x:c r="H86" s="21"/>
       <x:c r="I86" s="21"/>
-      <x:c r="J86" s="28"/>
+      <x:c r="J86" s="21"/>
       <x:c r="K86" s="21"/>
       <x:c r="L86" s="21"/>
       <x:c r="M86" s="21"/>
@@ -3673,7 +3566,7 @@
       <x:c r="AF86" s="21"/>
       <x:c r="AG86" s="21"/>
       <x:c r="AH86" s="21"/>
-      <x:c r="AI86"/>
+      <x:c r="AI86" s="21"/>
     </x:row>
     <x:row r="87" ht="23" customHeight="1">
       <x:c r="A87" s="21"/>
@@ -3685,7 +3578,7 @@
       <x:c r="G87" s="21"/>
       <x:c r="H87" s="21"/>
       <x:c r="I87" s="21"/>
-      <x:c r="J87" s="28"/>
+      <x:c r="J87" s="21"/>
       <x:c r="K87" s="21"/>
       <x:c r="L87" s="21"/>
       <x:c r="M87" s="21"/>
@@ -3710,7 +3603,7 @@
       <x:c r="AF87" s="21"/>
       <x:c r="AG87" s="21"/>
       <x:c r="AH87" s="21"/>
-      <x:c r="AI87"/>
+      <x:c r="AI87" s="21"/>
     </x:row>
     <x:row r="88" ht="23" customHeight="1">
       <x:c r="A88" s="21"/>
@@ -3722,7 +3615,7 @@
       <x:c r="G88" s="21"/>
       <x:c r="H88" s="21"/>
       <x:c r="I88" s="21"/>
-      <x:c r="J88" s="28"/>
+      <x:c r="J88" s="21"/>
       <x:c r="K88" s="21"/>
       <x:c r="L88" s="21"/>
       <x:c r="M88" s="21"/>
@@ -3747,7 +3640,7 @@
       <x:c r="AF88" s="21"/>
       <x:c r="AG88" s="21"/>
       <x:c r="AH88" s="21"/>
-      <x:c r="AI88"/>
+      <x:c r="AI88" s="21"/>
     </x:row>
     <x:row r="89" ht="23" customHeight="1">
       <x:c r="A89" s="21"/>
@@ -3759,7 +3652,7 @@
       <x:c r="G89" s="21"/>
       <x:c r="H89" s="21"/>
       <x:c r="I89" s="21"/>
-      <x:c r="J89" s="28"/>
+      <x:c r="J89" s="21"/>
       <x:c r="K89" s="21"/>
       <x:c r="L89" s="21"/>
       <x:c r="M89" s="21"/>
@@ -3784,7 +3677,7 @@
       <x:c r="AF89" s="21"/>
       <x:c r="AG89" s="21"/>
       <x:c r="AH89" s="21"/>
-      <x:c r="AI89"/>
+      <x:c r="AI89" s="21"/>
     </x:row>
     <x:row r="90" ht="23" customHeight="1">
       <x:c r="A90" s="21"/>
@@ -3796,7 +3689,7 @@
       <x:c r="G90" s="21"/>
       <x:c r="H90" s="21"/>
       <x:c r="I90" s="21"/>
-      <x:c r="J90" s="28"/>
+      <x:c r="J90" s="21"/>
       <x:c r="K90" s="21"/>
       <x:c r="L90" s="21"/>
       <x:c r="M90" s="21"/>
@@ -3821,7 +3714,7 @@
       <x:c r="AF90" s="21"/>
       <x:c r="AG90" s="21"/>
       <x:c r="AH90" s="21"/>
-      <x:c r="AI90"/>
+      <x:c r="AI90" s="21"/>
     </x:row>
     <x:row r="91" ht="23" customHeight="1">
       <x:c r="A91" s="21"/>
@@ -3833,7 +3726,7 @@
       <x:c r="G91" s="21"/>
       <x:c r="H91" s="21"/>
       <x:c r="I91" s="21"/>
-      <x:c r="J91" s="28"/>
+      <x:c r="J91" s="21"/>
       <x:c r="K91" s="21"/>
       <x:c r="L91" s="21"/>
       <x:c r="M91" s="21"/>
@@ -3858,7 +3751,7 @@
       <x:c r="AF91" s="21"/>
       <x:c r="AG91" s="21"/>
       <x:c r="AH91" s="21"/>
-      <x:c r="AI91"/>
+      <x:c r="AI91" s="21"/>
     </x:row>
     <x:row r="92" ht="23" customHeight="1">
       <x:c r="A92" s="21"/>
@@ -3870,7 +3763,7 @@
       <x:c r="G92" s="21"/>
       <x:c r="H92" s="21"/>
       <x:c r="I92" s="21"/>
-      <x:c r="J92" s="28"/>
+      <x:c r="J92" s="21"/>
       <x:c r="K92" s="21"/>
       <x:c r="L92" s="21"/>
       <x:c r="M92" s="21"/>
@@ -3895,7 +3788,7 @@
       <x:c r="AF92" s="21"/>
       <x:c r="AG92" s="21"/>
       <x:c r="AH92" s="21"/>
-      <x:c r="AI92"/>
+      <x:c r="AI92" s="21"/>
     </x:row>
     <x:row r="93" ht="23" customHeight="1">
       <x:c r="A93" s="21"/>
@@ -3907,7 +3800,7 @@
       <x:c r="G93" s="21"/>
       <x:c r="H93" s="21"/>
       <x:c r="I93" s="21"/>
-      <x:c r="J93" s="28"/>
+      <x:c r="J93" s="21"/>
       <x:c r="K93" s="21"/>
       <x:c r="L93" s="21"/>
       <x:c r="M93" s="21"/>
@@ -3932,7 +3825,7 @@
       <x:c r="AF93" s="21"/>
       <x:c r="AG93" s="21"/>
       <x:c r="AH93" s="21"/>
-      <x:c r="AI93"/>
+      <x:c r="AI93" s="21"/>
     </x:row>
     <x:row r="94" ht="23" customHeight="1">
       <x:c r="A94" s="21"/>
@@ -3944,7 +3837,7 @@
       <x:c r="G94" s="21"/>
       <x:c r="H94" s="21"/>
       <x:c r="I94" s="21"/>
-      <x:c r="J94" s="28"/>
+      <x:c r="J94" s="21"/>
       <x:c r="K94" s="21"/>
       <x:c r="L94" s="21"/>
       <x:c r="M94" s="21"/>
@@ -3969,7 +3862,7 @@
       <x:c r="AF94" s="21"/>
       <x:c r="AG94" s="21"/>
       <x:c r="AH94" s="21"/>
-      <x:c r="AI94"/>
+      <x:c r="AI94" s="21"/>
     </x:row>
     <x:row r="95" ht="23" customHeight="1">
       <x:c r="A95" s="21"/>
@@ -3981,7 +3874,7 @@
       <x:c r="G95" s="21"/>
       <x:c r="H95" s="21"/>
       <x:c r="I95" s="21"/>
-      <x:c r="J95" s="28"/>
+      <x:c r="J95" s="21"/>
       <x:c r="K95" s="21"/>
       <x:c r="L95" s="21"/>
       <x:c r="M95" s="21"/>
@@ -4006,7 +3899,7 @@
       <x:c r="AF95" s="21"/>
       <x:c r="AG95" s="21"/>
       <x:c r="AH95" s="21"/>
-      <x:c r="AI95"/>
+      <x:c r="AI95" s="21"/>
     </x:row>
     <x:row r="96" ht="23" customHeight="1">
       <x:c r="A96" s="21"/>
@@ -4018,7 +3911,7 @@
       <x:c r="G96" s="21"/>
       <x:c r="H96" s="21"/>
       <x:c r="I96" s="21"/>
-      <x:c r="J96" s="28"/>
+      <x:c r="J96" s="21"/>
       <x:c r="K96" s="21"/>
       <x:c r="L96" s="21"/>
       <x:c r="M96" s="21"/>
@@ -4043,7 +3936,7 @@
       <x:c r="AF96" s="21"/>
       <x:c r="AG96" s="21"/>
       <x:c r="AH96" s="21"/>
-      <x:c r="AI96"/>
+      <x:c r="AI96" s="21"/>
     </x:row>
     <x:row r="97" ht="23" customHeight="1">
       <x:c r="A97" s="21"/>
@@ -4055,7 +3948,7 @@
       <x:c r="G97" s="21"/>
       <x:c r="H97" s="21"/>
       <x:c r="I97" s="21"/>
-      <x:c r="J97" s="28"/>
+      <x:c r="J97" s="21"/>
       <x:c r="K97" s="21"/>
       <x:c r="L97" s="21"/>
       <x:c r="M97" s="21"/>
@@ -4080,7 +3973,7 @@
       <x:c r="AF97" s="21"/>
       <x:c r="AG97" s="21"/>
       <x:c r="AH97" s="21"/>
-      <x:c r="AI97"/>
+      <x:c r="AI97" s="21"/>
     </x:row>
     <x:row r="98" ht="23" customHeight="1">
       <x:c r="A98" s="21"/>
@@ -4092,7 +3985,7 @@
       <x:c r="G98" s="21"/>
       <x:c r="H98" s="21"/>
       <x:c r="I98" s="21"/>
-      <x:c r="J98" s="28"/>
+      <x:c r="J98" s="21"/>
       <x:c r="K98" s="21"/>
       <x:c r="L98" s="21"/>
       <x:c r="M98" s="21"/>
@@ -4117,7 +4010,7 @@
       <x:c r="AF98" s="21"/>
       <x:c r="AG98" s="21"/>
       <x:c r="AH98" s="21"/>
-      <x:c r="AI98"/>
+      <x:c r="AI98" s="21"/>
     </x:row>
     <x:row r="99" ht="23" customHeight="1">
       <x:c r="A99" s="21"/>
@@ -4129,7 +4022,7 @@
       <x:c r="G99" s="21"/>
       <x:c r="H99" s="21"/>
       <x:c r="I99" s="21"/>
-      <x:c r="J99" s="28"/>
+      <x:c r="J99" s="21"/>
       <x:c r="K99" s="21"/>
       <x:c r="L99" s="21"/>
       <x:c r="M99" s="21"/>
@@ -4154,7 +4047,7 @@
       <x:c r="AF99" s="21"/>
       <x:c r="AG99" s="21"/>
       <x:c r="AH99" s="21"/>
-      <x:c r="AI99"/>
+      <x:c r="AI99" s="21"/>
     </x:row>
     <x:row r="100" ht="23" customHeight="1">
       <x:c r="A100" s="21"/>
@@ -4166,7 +4059,7 @@
       <x:c r="G100" s="21"/>
       <x:c r="H100" s="21"/>
       <x:c r="I100" s="21"/>
-      <x:c r="J100" s="28"/>
+      <x:c r="J100" s="21"/>
       <x:c r="K100" s="21"/>
       <x:c r="L100" s="21"/>
       <x:c r="M100" s="21"/>
@@ -4191,7 +4084,7 @@
       <x:c r="AF100" s="21"/>
       <x:c r="AG100" s="21"/>
       <x:c r="AH100" s="21"/>
-      <x:c r="AI100"/>
+      <x:c r="AI100" s="21"/>
     </x:row>
     <x:row r="101" ht="23" customHeight="1">
       <x:c r="A101" s="21"/>
@@ -4203,7 +4096,7 @@
       <x:c r="G101" s="21"/>
       <x:c r="H101" s="21"/>
       <x:c r="I101" s="21"/>
-      <x:c r="J101" s="28"/>
+      <x:c r="J101" s="21"/>
       <x:c r="K101" s="21"/>
       <x:c r="L101" s="21"/>
       <x:c r="M101" s="21"/>
@@ -4228,7 +4121,7 @@
       <x:c r="AF101" s="21"/>
       <x:c r="AG101" s="21"/>
       <x:c r="AH101" s="21"/>
-      <x:c r="AI101"/>
+      <x:c r="AI101" s="21"/>
     </x:row>
     <x:row r="102" ht="23" customHeight="1">
       <x:c r="A102" s="21"/>
@@ -4240,7 +4133,7 @@
       <x:c r="G102" s="21"/>
       <x:c r="H102" s="21"/>
       <x:c r="I102" s="21"/>
-      <x:c r="J102" s="28"/>
+      <x:c r="J102" s="21"/>
       <x:c r="K102" s="21"/>
       <x:c r="L102" s="21"/>
       <x:c r="M102" s="21"/>
@@ -4265,7 +4158,7 @@
       <x:c r="AF102" s="21"/>
       <x:c r="AG102" s="21"/>
       <x:c r="AH102" s="21"/>
-      <x:c r="AI102"/>
+      <x:c r="AI102" s="21"/>
     </x:row>
     <x:row r="103" ht="23" customHeight="1">
       <x:c r="A103" s="21"/>
@@ -4277,7 +4170,7 @@
       <x:c r="G103" s="21"/>
       <x:c r="H103" s="21"/>
       <x:c r="I103" s="21"/>
-      <x:c r="J103" s="28"/>
+      <x:c r="J103" s="21"/>
       <x:c r="K103" s="21"/>
       <x:c r="L103" s="21"/>
       <x:c r="M103" s="21"/>
@@ -4302,7 +4195,7 @@
       <x:c r="AF103" s="21"/>
       <x:c r="AG103" s="21"/>
       <x:c r="AH103" s="21"/>
-      <x:c r="AI103"/>
+      <x:c r="AI103" s="21"/>
     </x:row>
     <x:row r="104" ht="23" customHeight="1">
       <x:c r="A104" s="21"/>
@@ -4314,7 +4207,7 @@
       <x:c r="G104" s="21"/>
       <x:c r="H104" s="21"/>
       <x:c r="I104" s="21"/>
-      <x:c r="J104" s="28"/>
+      <x:c r="J104" s="21"/>
       <x:c r="K104" s="21"/>
       <x:c r="L104" s="21"/>
       <x:c r="M104" s="21"/>
@@ -4339,7 +4232,7 @@
       <x:c r="AF104" s="21"/>
       <x:c r="AG104" s="21"/>
       <x:c r="AH104" s="21"/>
-      <x:c r="AI104"/>
+      <x:c r="AI104" s="21"/>
     </x:row>
     <x:row r="105" ht="23" customHeight="1">
       <x:c r="A105" s="21"/>
@@ -4351,7 +4244,7 @@
       <x:c r="G105" s="21"/>
       <x:c r="H105" s="21"/>
       <x:c r="I105" s="21"/>
-      <x:c r="J105" s="28"/>
+      <x:c r="J105" s="21"/>
       <x:c r="K105" s="21"/>
       <x:c r="L105" s="21"/>
       <x:c r="M105" s="21"/>
@@ -4376,7 +4269,7 @@
       <x:c r="AF105" s="21"/>
       <x:c r="AG105" s="21"/>
       <x:c r="AH105" s="21"/>
-      <x:c r="AI105"/>
+      <x:c r="AI105" s="21"/>
     </x:row>
     <x:row r="106" ht="23" customHeight="1">
       <x:c r="A106" s="21"/>
@@ -4388,7 +4281,7 @@
       <x:c r="G106" s="21"/>
       <x:c r="H106" s="21"/>
       <x:c r="I106" s="21"/>
-      <x:c r="J106" s="28"/>
+      <x:c r="J106" s="21"/>
       <x:c r="K106" s="21"/>
       <x:c r="L106" s="21"/>
       <x:c r="M106" s="21"/>
@@ -4413,7 +4306,7 @@
       <x:c r="AF106" s="21"/>
       <x:c r="AG106" s="21"/>
       <x:c r="AH106" s="21"/>
-      <x:c r="AI106"/>
+      <x:c r="AI106" s="21"/>
     </x:row>
     <x:row r="107" ht="23" customHeight="1">
       <x:c r="A107" s="21"/>
@@ -4425,7 +4318,7 @@
       <x:c r="G107" s="21"/>
       <x:c r="H107" s="21"/>
       <x:c r="I107" s="21"/>
-      <x:c r="J107" s="28"/>
+      <x:c r="J107" s="21"/>
       <x:c r="K107" s="21"/>
       <x:c r="L107" s="21"/>
       <x:c r="M107" s="21"/>
@@ -4450,7 +4343,7 @@
       <x:c r="AF107" s="21"/>
       <x:c r="AG107" s="21"/>
       <x:c r="AH107" s="21"/>
-      <x:c r="AI107"/>
+      <x:c r="AI107" s="21"/>
     </x:row>
     <x:row r="108" ht="23" customHeight="1">
       <x:c r="A108" s="21"/>
@@ -4462,7 +4355,7 @@
       <x:c r="G108" s="21"/>
       <x:c r="H108" s="21"/>
       <x:c r="I108" s="21"/>
-      <x:c r="J108" s="28"/>
+      <x:c r="J108" s="21"/>
       <x:c r="K108" s="21"/>
       <x:c r="L108" s="21"/>
       <x:c r="M108" s="21"/>
@@ -4487,7 +4380,7 @@
       <x:c r="AF108" s="21"/>
       <x:c r="AG108" s="21"/>
       <x:c r="AH108" s="21"/>
-      <x:c r="AI108"/>
+      <x:c r="AI108" s="21"/>
     </x:row>
     <x:row r="109" ht="23" customHeight="1">
       <x:c r="A109" s="21"/>
@@ -4499,7 +4392,7 @@
       <x:c r="G109" s="21"/>
       <x:c r="H109" s="21"/>
       <x:c r="I109" s="21"/>
-      <x:c r="J109" s="28"/>
+      <x:c r="J109" s="21"/>
       <x:c r="K109" s="21"/>
       <x:c r="L109" s="21"/>
       <x:c r="M109" s="21"/>
@@ -4524,7 +4417,7 @@
       <x:c r="AF109" s="21"/>
       <x:c r="AG109" s="21"/>
       <x:c r="AH109" s="21"/>
-      <x:c r="AI109"/>
+      <x:c r="AI109" s="21"/>
     </x:row>
     <x:row r="110" ht="23" customHeight="1">
       <x:c r="A110" s="21"/>
@@ -4536,7 +4429,7 @@
       <x:c r="G110" s="21"/>
       <x:c r="H110" s="21"/>
       <x:c r="I110" s="21"/>
-      <x:c r="J110" s="28"/>
+      <x:c r="J110" s="21"/>
       <x:c r="K110" s="21"/>
       <x:c r="L110" s="21"/>
       <x:c r="M110" s="21"/>
@@ -4561,7 +4454,7 @@
       <x:c r="AF110" s="21"/>
       <x:c r="AG110" s="21"/>
       <x:c r="AH110" s="21"/>
-      <x:c r="AI110"/>
+      <x:c r="AI110" s="21"/>
     </x:row>
     <x:row r="111" ht="23" customHeight="1">
       <x:c r="A111" s="21"/>
@@ -4573,7 +4466,7 @@
       <x:c r="G111" s="21"/>
       <x:c r="H111" s="21"/>
       <x:c r="I111" s="21"/>
-      <x:c r="J111" s="28"/>
+      <x:c r="J111" s="21"/>
       <x:c r="K111" s="21"/>
       <x:c r="L111" s="21"/>
       <x:c r="M111" s="21"/>
@@ -4598,7 +4491,7 @@
       <x:c r="AF111" s="21"/>
       <x:c r="AG111" s="21"/>
       <x:c r="AH111" s="21"/>
-      <x:c r="AI111"/>
+      <x:c r="AI111" s="21"/>
     </x:row>
     <x:row r="112" ht="23" customHeight="1">
       <x:c r="A112" s="21"/>
@@ -4610,7 +4503,7 @@
       <x:c r="G112" s="21"/>
       <x:c r="H112" s="21"/>
       <x:c r="I112" s="21"/>
-      <x:c r="J112" s="28"/>
+      <x:c r="J112" s="21"/>
       <x:c r="K112" s="21"/>
       <x:c r="L112" s="21"/>
       <x:c r="M112" s="21"/>
@@ -4635,7 +4528,7 @@
       <x:c r="AF112" s="21"/>
       <x:c r="AG112" s="21"/>
       <x:c r="AH112" s="21"/>
-      <x:c r="AI112"/>
+      <x:c r="AI112" s="21"/>
     </x:row>
     <x:row r="113" ht="23" customHeight="1">
       <x:c r="A113" s="21"/>
@@ -4647,7 +4540,7 @@
       <x:c r="G113" s="21"/>
       <x:c r="H113" s="21"/>
       <x:c r="I113" s="21"/>
-      <x:c r="J113" s="28"/>
+      <x:c r="J113" s="21"/>
       <x:c r="K113" s="21"/>
       <x:c r="L113" s="21"/>
       <x:c r="M113" s="21"/>
@@ -4672,7 +4565,7 @@
       <x:c r="AF113" s="21"/>
       <x:c r="AG113" s="21"/>
       <x:c r="AH113" s="21"/>
-      <x:c r="AI113"/>
+      <x:c r="AI113" s="21"/>
     </x:row>
     <x:row r="114" ht="23" customHeight="1">
       <x:c r="A114" s="21"/>
@@ -4684,7 +4577,7 @@
       <x:c r="G114" s="21"/>
       <x:c r="H114" s="21"/>
       <x:c r="I114" s="21"/>
-      <x:c r="J114" s="28"/>
+      <x:c r="J114" s="21"/>
       <x:c r="K114" s="21"/>
       <x:c r="L114" s="21"/>
       <x:c r="M114" s="21"/>
@@ -4709,7 +4602,7 @@
       <x:c r="AF114" s="21"/>
       <x:c r="AG114" s="21"/>
       <x:c r="AH114" s="21"/>
-      <x:c r="AI114"/>
+      <x:c r="AI114" s="21"/>
     </x:row>
     <x:row r="115" ht="23" customHeight="1">
       <x:c r="A115" s="21"/>
@@ -4721,7 +4614,7 @@
       <x:c r="G115" s="21"/>
       <x:c r="H115" s="21"/>
       <x:c r="I115" s="21"/>
-      <x:c r="J115" s="28"/>
+      <x:c r="J115" s="21"/>
       <x:c r="K115" s="21"/>
       <x:c r="L115" s="21"/>
       <x:c r="M115" s="21"/>
@@ -4746,7 +4639,7 @@
       <x:c r="AF115" s="21"/>
       <x:c r="AG115" s="21"/>
       <x:c r="AH115" s="21"/>
-      <x:c r="AI115"/>
+      <x:c r="AI115" s="21"/>
     </x:row>
     <x:row r="116" ht="23" customHeight="1">
       <x:c r="A116" s="21"/>
@@ -4758,7 +4651,7 @@
       <x:c r="G116" s="21"/>
       <x:c r="H116" s="21"/>
       <x:c r="I116" s="21"/>
-      <x:c r="J116" s="28"/>
+      <x:c r="J116" s="21"/>
       <x:c r="K116" s="21"/>
       <x:c r="L116" s="21"/>
       <x:c r="M116" s="21"/>
@@ -4783,7 +4676,7 @@
       <x:c r="AF116" s="21"/>
       <x:c r="AG116" s="21"/>
       <x:c r="AH116" s="21"/>
-      <x:c r="AI116"/>
+      <x:c r="AI116" s="21"/>
     </x:row>
     <x:row r="117" ht="23" customHeight="1">
       <x:c r="A117" s="21"/>
@@ -4795,7 +4688,7 @@
       <x:c r="G117" s="21"/>
       <x:c r="H117" s="21"/>
       <x:c r="I117" s="21"/>
-      <x:c r="J117" s="28"/>
+      <x:c r="J117" s="21"/>
       <x:c r="K117" s="21"/>
       <x:c r="L117" s="21"/>
       <x:c r="M117" s="21"/>
@@ -4820,7 +4713,7 @@
       <x:c r="AF117" s="21"/>
       <x:c r="AG117" s="21"/>
       <x:c r="AH117" s="21"/>
-      <x:c r="AI117"/>
+      <x:c r="AI117" s="21"/>
     </x:row>
     <x:row r="118" ht="23" customHeight="1">
       <x:c r="A118" s="21"/>
@@ -4832,7 +4725,7 @@
       <x:c r="G118" s="21"/>
       <x:c r="H118" s="21"/>
       <x:c r="I118" s="21"/>
-      <x:c r="J118" s="28"/>
+      <x:c r="J118" s="21"/>
       <x:c r="K118" s="21"/>
       <x:c r="L118" s="21"/>
       <x:c r="M118" s="21"/>
@@ -4857,7 +4750,7 @@
       <x:c r="AF118" s="21"/>
       <x:c r="AG118" s="21"/>
       <x:c r="AH118" s="21"/>
-      <x:c r="AI118"/>
+      <x:c r="AI118" s="21"/>
     </x:row>
     <x:row r="119" ht="23" customHeight="1">
       <x:c r="A119" s="21"/>
@@ -4869,7 +4762,7 @@
       <x:c r="G119" s="21"/>
       <x:c r="H119" s="21"/>
       <x:c r="I119" s="21"/>
-      <x:c r="J119" s="28"/>
+      <x:c r="J119" s="21"/>
       <x:c r="K119" s="21"/>
       <x:c r="L119" s="21"/>
       <x:c r="M119" s="21"/>
@@ -4894,7 +4787,7 @@
       <x:c r="AF119" s="21"/>
       <x:c r="AG119" s="21"/>
       <x:c r="AH119" s="21"/>
-      <x:c r="AI119"/>
+      <x:c r="AI119" s="21"/>
     </x:row>
     <x:row r="120" ht="23" customHeight="1">
       <x:c r="A120" s="21"/>
@@ -4906,7 +4799,7 @@
       <x:c r="G120" s="21"/>
       <x:c r="H120" s="21"/>
       <x:c r="I120" s="21"/>
-      <x:c r="J120" s="28"/>
+      <x:c r="J120" s="21"/>
       <x:c r="K120" s="21"/>
       <x:c r="L120" s="21"/>
       <x:c r="M120" s="21"/>
@@ -4931,7 +4824,7 @@
       <x:c r="AF120" s="21"/>
       <x:c r="AG120" s="21"/>
       <x:c r="AH120" s="21"/>
-      <x:c r="AI120"/>
+      <x:c r="AI120" s="21"/>
     </x:row>
     <x:row r="121" ht="23" customHeight="1">
       <x:c r="A121" s="21"/>
@@ -4943,7 +4836,7 @@
       <x:c r="G121" s="21"/>
       <x:c r="H121" s="21"/>
       <x:c r="I121" s="21"/>
-      <x:c r="J121" s="28"/>
+      <x:c r="J121" s="21"/>
       <x:c r="K121" s="21"/>
       <x:c r="L121" s="21"/>
       <x:c r="M121" s="21"/>
@@ -4968,7 +4861,7 @@
       <x:c r="AF121" s="21"/>
       <x:c r="AG121" s="21"/>
       <x:c r="AH121" s="21"/>
-      <x:c r="AI121"/>
+      <x:c r="AI121" s="21"/>
     </x:row>
     <x:row r="122" ht="23" customHeight="1">
       <x:c r="A122" s="21"/>
@@ -4980,7 +4873,7 @@
       <x:c r="G122" s="21"/>
       <x:c r="H122" s="21"/>
       <x:c r="I122" s="21"/>
-      <x:c r="J122" s="28"/>
+      <x:c r="J122" s="21"/>
       <x:c r="K122" s="21"/>
       <x:c r="L122" s="21"/>
       <x:c r="M122" s="21"/>
@@ -5005,7 +4898,7 @@
       <x:c r="AF122" s="21"/>
       <x:c r="AG122" s="21"/>
       <x:c r="AH122" s="21"/>
-      <x:c r="AI122"/>
+      <x:c r="AI122" s="21"/>
     </x:row>
     <x:row r="123" ht="23" customHeight="1">
       <x:c r="A123" s="21"/>
@@ -5017,7 +4910,7 @@
       <x:c r="G123" s="21"/>
       <x:c r="H123" s="21"/>
       <x:c r="I123" s="21"/>
-      <x:c r="J123" s="28"/>
+      <x:c r="J123" s="21"/>
       <x:c r="K123" s="21"/>
       <x:c r="L123" s="21"/>
       <x:c r="M123" s="21"/>
@@ -5042,7 +4935,7 @@
       <x:c r="AF123" s="21"/>
       <x:c r="AG123" s="21"/>
       <x:c r="AH123" s="21"/>
-      <x:c r="AI123"/>
+      <x:c r="AI123" s="21"/>
     </x:row>
     <x:row r="124" ht="23" customHeight="1">
       <x:c r="A124" s="21"/>
@@ -5054,7 +4947,7 @@
       <x:c r="G124" s="21"/>
       <x:c r="H124" s="21"/>
       <x:c r="I124" s="21"/>
-      <x:c r="J124" s="28"/>
+      <x:c r="J124" s="21"/>
       <x:c r="K124" s="21"/>
       <x:c r="L124" s="21"/>
       <x:c r="M124" s="21"/>
@@ -5079,7 +4972,7 @@
       <x:c r="AF124" s="21"/>
       <x:c r="AG124" s="21"/>
       <x:c r="AH124" s="21"/>
-      <x:c r="AI124"/>
+      <x:c r="AI124" s="21"/>
     </x:row>
     <x:row r="125" ht="23" customHeight="1">
       <x:c r="A125" s="21"/>
@@ -5091,7 +4984,7 @@
       <x:c r="G125" s="21"/>
       <x:c r="H125" s="21"/>
       <x:c r="I125" s="21"/>
-      <x:c r="J125" s="28"/>
+      <x:c r="J125" s="21"/>
       <x:c r="K125" s="21"/>
       <x:c r="L125" s="21"/>
       <x:c r="M125" s="21"/>
@@ -5116,7 +5009,7 @@
       <x:c r="AF125" s="21"/>
       <x:c r="AG125" s="21"/>
       <x:c r="AH125" s="21"/>
-      <x:c r="AI125"/>
+      <x:c r="AI125" s="21"/>
     </x:row>
     <x:row r="126" ht="23" customHeight="1">
       <x:c r="A126" s="21"/>
@@ -5128,7 +5021,7 @@
       <x:c r="G126" s="21"/>
       <x:c r="H126" s="21"/>
       <x:c r="I126" s="21"/>
-      <x:c r="J126" s="28"/>
+      <x:c r="J126" s="21"/>
       <x:c r="K126" s="21"/>
       <x:c r="L126" s="21"/>
       <x:c r="M126" s="21"/>
@@ -5153,7 +5046,7 @@
       <x:c r="AF126" s="21"/>
       <x:c r="AG126" s="21"/>
       <x:c r="AH126" s="21"/>
-      <x:c r="AI126"/>
+      <x:c r="AI126" s="21"/>
     </x:row>
     <x:row r="127" ht="23" customHeight="1">
       <x:c r="A127" s="21"/>
@@ -5165,7 +5058,7 @@
       <x:c r="G127" s="21"/>
       <x:c r="H127" s="21"/>
       <x:c r="I127" s="21"/>
-      <x:c r="J127" s="28"/>
+      <x:c r="J127" s="21"/>
       <x:c r="K127" s="21"/>
       <x:c r="L127" s="21"/>
       <x:c r="M127" s="21"/>
@@ -5190,7 +5083,7 @@
       <x:c r="AF127" s="21"/>
       <x:c r="AG127" s="21"/>
       <x:c r="AH127" s="21"/>
-      <x:c r="AI127"/>
+      <x:c r="AI127" s="21"/>
     </x:row>
     <x:row r="128" ht="23" customHeight="1">
       <x:c r="A128" s="21"/>
@@ -5202,7 +5095,7 @@
       <x:c r="G128" s="21"/>
       <x:c r="H128" s="21"/>
       <x:c r="I128" s="21"/>
-      <x:c r="J128" s="28"/>
+      <x:c r="J128" s="21"/>
       <x:c r="K128" s="21"/>
       <x:c r="L128" s="21"/>
       <x:c r="M128" s="21"/>
@@ -5227,7 +5120,7 @@
       <x:c r="AF128" s="21"/>
       <x:c r="AG128" s="21"/>
       <x:c r="AH128" s="21"/>
-      <x:c r="AI128"/>
+      <x:c r="AI128" s="21"/>
     </x:row>
     <x:row r="129" ht="23" customHeight="1">
       <x:c r="A129" s="21"/>
@@ -5239,7 +5132,7 @@
       <x:c r="G129" s="21"/>
       <x:c r="H129" s="21"/>
       <x:c r="I129" s="21"/>
-      <x:c r="J129" s="28"/>
+      <x:c r="J129" s="21"/>
       <x:c r="K129" s="21"/>
       <x:c r="L129" s="21"/>
       <x:c r="M129" s="21"/>
@@ -5264,7 +5157,7 @@
       <x:c r="AF129" s="21"/>
       <x:c r="AG129" s="21"/>
       <x:c r="AH129" s="21"/>
-      <x:c r="AI129"/>
+      <x:c r="AI129" s="21"/>
     </x:row>
     <x:row r="130" ht="23" customHeight="1">
       <x:c r="A130" s="21"/>
@@ -5276,7 +5169,7 @@
       <x:c r="G130" s="21"/>
       <x:c r="H130" s="21"/>
       <x:c r="I130" s="21"/>
-      <x:c r="J130" s="28"/>
+      <x:c r="J130" s="21"/>
       <x:c r="K130" s="21"/>
       <x:c r="L130" s="21"/>
       <x:c r="M130" s="21"/>
@@ -5301,7 +5194,7 @@
       <x:c r="AF130" s="21"/>
       <x:c r="AG130" s="21"/>
       <x:c r="AH130" s="21"/>
-      <x:c r="AI130"/>
+      <x:c r="AI130" s="21"/>
     </x:row>
     <x:row r="131" ht="23" customHeight="1">
       <x:c r="A131" s="21"/>
@@ -5313,7 +5206,7 @@
       <x:c r="G131" s="21"/>
       <x:c r="H131" s="21"/>
       <x:c r="I131" s="21"/>
-      <x:c r="J131" s="28"/>
+      <x:c r="J131" s="21"/>
       <x:c r="K131" s="21"/>
       <x:c r="L131" s="21"/>
       <x:c r="M131" s="21"/>
@@ -5338,7 +5231,7 @@
       <x:c r="AF131" s="21"/>
       <x:c r="AG131" s="21"/>
       <x:c r="AH131" s="21"/>
-      <x:c r="AI131"/>
+      <x:c r="AI131" s="21"/>
     </x:row>
     <x:row r="132" ht="23" customHeight="1">
       <x:c r="A132" s="21"/>
@@ -5350,7 +5243,7 @@
       <x:c r="G132" s="21"/>
       <x:c r="H132" s="21"/>
       <x:c r="I132" s="21"/>
-      <x:c r="J132" s="28"/>
+      <x:c r="J132" s="21"/>
       <x:c r="K132" s="21"/>
       <x:c r="L132" s="21"/>
       <x:c r="M132" s="21"/>
@@ -5375,7 +5268,7 @@
       <x:c r="AF132" s="21"/>
       <x:c r="AG132" s="21"/>
       <x:c r="AH132" s="21"/>
-      <x:c r="AI132"/>
+      <x:c r="AI132" s="21"/>
     </x:row>
     <x:row r="133" ht="23" customHeight="1">
       <x:c r="A133" s="21"/>
@@ -5387,7 +5280,7 @@
       <x:c r="G133" s="21"/>
       <x:c r="H133" s="21"/>
       <x:c r="I133" s="21"/>
-      <x:c r="J133" s="28"/>
+      <x:c r="J133" s="21"/>
       <x:c r="K133" s="21"/>
       <x:c r="L133" s="21"/>
       <x:c r="M133" s="21"/>
@@ -5412,7 +5305,7 @@
       <x:c r="AF133" s="21"/>
       <x:c r="AG133" s="21"/>
       <x:c r="AH133" s="21"/>
-      <x:c r="AI133"/>
+      <x:c r="AI133" s="21"/>
     </x:row>
     <x:row r="134" ht="23" customHeight="1">
       <x:c r="A134" s="21"/>
@@ -5424,7 +5317,7 @@
       <x:c r="G134" s="21"/>
       <x:c r="H134" s="21"/>
       <x:c r="I134" s="21"/>
-      <x:c r="J134" s="28"/>
+      <x:c r="J134" s="21"/>
       <x:c r="K134" s="21"/>
       <x:c r="L134" s="21"/>
       <x:c r="M134" s="21"/>
@@ -5449,7 +5342,7 @@
       <x:c r="AF134" s="21"/>
       <x:c r="AG134" s="21"/>
       <x:c r="AH134" s="21"/>
-      <x:c r="AI134"/>
+      <x:c r="AI134" s="21"/>
     </x:row>
     <x:row r="135" ht="23" customHeight="1">
       <x:c r="A135" s="21"/>
@@ -5461,7 +5354,7 @@
       <x:c r="G135" s="21"/>
       <x:c r="H135" s="21"/>
       <x:c r="I135" s="21"/>
-      <x:c r="J135" s="28"/>
+      <x:c r="J135" s="21"/>
       <x:c r="K135" s="21"/>
       <x:c r="L135" s="21"/>
       <x:c r="M135" s="21"/>
@@ -5486,7 +5379,7 @@
       <x:c r="AF135" s="21"/>
       <x:c r="AG135" s="21"/>
       <x:c r="AH135" s="21"/>
-      <x:c r="AI135"/>
+      <x:c r="AI135" s="21"/>
     </x:row>
     <x:row r="136" ht="23" customHeight="1">
       <x:c r="A136" s="21"/>
@@ -5498,7 +5391,7 @@
       <x:c r="G136" s="21"/>
       <x:c r="H136" s="21"/>
       <x:c r="I136" s="21"/>
-      <x:c r="J136" s="28"/>
+      <x:c r="J136" s="21"/>
       <x:c r="K136" s="21"/>
       <x:c r="L136" s="21"/>
       <x:c r="M136" s="21"/>
@@ -5523,7 +5416,7 @@
       <x:c r="AF136" s="21"/>
       <x:c r="AG136" s="21"/>
       <x:c r="AH136" s="21"/>
-      <x:c r="AI136"/>
+      <x:c r="AI136" s="21"/>
     </x:row>
     <x:row r="137" ht="23" customHeight="1">
       <x:c r="A137" s="21"/>
@@ -5535,7 +5428,7 @@
       <x:c r="G137" s="21"/>
       <x:c r="H137" s="21"/>
       <x:c r="I137" s="21"/>
-      <x:c r="J137" s="28"/>
+      <x:c r="J137" s="21"/>
       <x:c r="K137" s="21"/>
       <x:c r="L137" s="21"/>
       <x:c r="M137" s="21"/>
@@ -5560,7 +5453,7 @@
       <x:c r="AF137" s="21"/>
       <x:c r="AG137" s="21"/>
       <x:c r="AH137" s="21"/>
-      <x:c r="AI137"/>
+      <x:c r="AI137" s="21"/>
     </x:row>
     <x:row r="138" ht="23" customHeight="1">
       <x:c r="A138" s="21"/>
@@ -5572,7 +5465,7 @@
       <x:c r="G138" s="21"/>
       <x:c r="H138" s="21"/>
       <x:c r="I138" s="21"/>
-      <x:c r="J138" s="28"/>
+      <x:c r="J138" s="21"/>
       <x:c r="K138" s="21"/>
       <x:c r="L138" s="21"/>
       <x:c r="M138" s="21"/>
@@ -5597,7 +5490,7 @@
       <x:c r="AF138" s="21"/>
       <x:c r="AG138" s="21"/>
       <x:c r="AH138" s="21"/>
-      <x:c r="AI138"/>
+      <x:c r="AI138" s="21"/>
     </x:row>
     <x:row r="139" ht="23" customHeight="1">
       <x:c r="A139" s="21"/>
@@ -5609,7 +5502,7 @@
       <x:c r="G139" s="21"/>
       <x:c r="H139" s="21"/>
       <x:c r="I139" s="21"/>
-      <x:c r="J139" s="28"/>
+      <x:c r="J139" s="21"/>
       <x:c r="K139" s="21"/>
       <x:c r="L139" s="21"/>
       <x:c r="M139" s="21"/>
@@ -5634,7 +5527,7 @@
       <x:c r="AF139" s="21"/>
       <x:c r="AG139" s="21"/>
       <x:c r="AH139" s="21"/>
-      <x:c r="AI139"/>
+      <x:c r="AI139" s="21"/>
     </x:row>
     <x:row r="140" ht="23" customHeight="1">
       <x:c r="A140" s="21"/>
@@ -5646,7 +5539,7 @@
       <x:c r="G140" s="21"/>
       <x:c r="H140" s="21"/>
       <x:c r="I140" s="21"/>
-      <x:c r="J140" s="28"/>
+      <x:c r="J140" s="21"/>
       <x:c r="K140" s="21"/>
       <x:c r="L140" s="21"/>
       <x:c r="M140" s="21"/>
@@ -5671,7 +5564,7 @@
       <x:c r="AF140" s="21"/>
       <x:c r="AG140" s="21"/>
       <x:c r="AH140" s="21"/>
-      <x:c r="AI140"/>
+      <x:c r="AI140" s="21"/>
     </x:row>
     <x:row r="141" ht="23" customHeight="1">
       <x:c r="A141" s="21"/>
@@ -5683,7 +5576,7 @@
       <x:c r="G141" s="21"/>
       <x:c r="H141" s="21"/>
       <x:c r="I141" s="21"/>
-      <x:c r="J141" s="28"/>
+      <x:c r="J141" s="21"/>
       <x:c r="K141" s="21"/>
       <x:c r="L141" s="21"/>
       <x:c r="M141" s="21"/>
@@ -5708,7 +5601,7 @@
       <x:c r="AF141" s="21"/>
       <x:c r="AG141" s="21"/>
       <x:c r="AH141" s="21"/>
-      <x:c r="AI141"/>
+      <x:c r="AI141" s="21"/>
     </x:row>
     <x:row r="142" ht="23" customHeight="1">
       <x:c r="A142" s="21"/>
@@ -5720,7 +5613,7 @@
       <x:c r="G142" s="21"/>
       <x:c r="H142" s="21"/>
       <x:c r="I142" s="21"/>
-      <x:c r="J142" s="28"/>
+      <x:c r="J142" s="21"/>
       <x:c r="K142" s="21"/>
       <x:c r="L142" s="21"/>
       <x:c r="M142" s="21"/>
@@ -5745,7 +5638,7 @@
       <x:c r="AF142" s="21"/>
       <x:c r="AG142" s="21"/>
       <x:c r="AH142" s="21"/>
-      <x:c r="AI142"/>
+      <x:c r="AI142" s="21"/>
     </x:row>
     <x:row r="143" ht="23" customHeight="1">
       <x:c r="A143" s="21"/>
@@ -5757,7 +5650,7 @@
       <x:c r="G143" s="21"/>
       <x:c r="H143" s="21"/>
       <x:c r="I143" s="21"/>
-      <x:c r="J143" s="28"/>
+      <x:c r="J143" s="21"/>
       <x:c r="K143" s="21"/>
       <x:c r="L143" s="21"/>
       <x:c r="M143" s="21"/>
@@ -5782,7 +5675,7 @@
       <x:c r="AF143" s="21"/>
       <x:c r="AG143" s="21"/>
       <x:c r="AH143" s="21"/>
-      <x:c r="AI143"/>
+      <x:c r="AI143" s="21"/>
     </x:row>
     <x:row r="144" ht="23" customHeight="1">
       <x:c r="A144" s="21"/>
@@ -5794,7 +5687,7 @@
       <x:c r="G144" s="21"/>
       <x:c r="H144" s="21"/>
       <x:c r="I144" s="21"/>
-      <x:c r="J144" s="28"/>
+      <x:c r="J144" s="21"/>
       <x:c r="K144" s="21"/>
       <x:c r="L144" s="21"/>
       <x:c r="M144" s="21"/>
@@ -5819,7 +5712,7 @@
       <x:c r="AF144" s="21"/>
       <x:c r="AG144" s="21"/>
       <x:c r="AH144" s="21"/>
-      <x:c r="AI144"/>
+      <x:c r="AI144" s="21"/>
     </x:row>
     <x:row r="145" ht="23" customHeight="1">
       <x:c r="A145" s="21"/>
@@ -5831,7 +5724,7 @@
       <x:c r="G145" s="21"/>
       <x:c r="H145" s="21"/>
       <x:c r="I145" s="21"/>
-      <x:c r="J145" s="28"/>
+      <x:c r="J145" s="21"/>
       <x:c r="K145" s="21"/>
       <x:c r="L145" s="21"/>
       <x:c r="M145" s="21"/>
@@ -5856,7 +5749,7 @@
       <x:c r="AF145" s="21"/>
       <x:c r="AG145" s="21"/>
       <x:c r="AH145" s="21"/>
-      <x:c r="AI145"/>
+      <x:c r="AI145" s="21"/>
     </x:row>
     <x:row r="146" ht="23" customHeight="1">
       <x:c r="A146" s="21"/>
@@ -5868,7 +5761,7 @@
       <x:c r="G146" s="21"/>
       <x:c r="H146" s="21"/>
       <x:c r="I146" s="21"/>
-      <x:c r="J146" s="28"/>
+      <x:c r="J146" s="21"/>
       <x:c r="K146" s="21"/>
       <x:c r="L146" s="21"/>
       <x:c r="M146" s="21"/>
@@ -5893,7 +5786,7 @@
       <x:c r="AF146" s="21"/>
       <x:c r="AG146" s="21"/>
       <x:c r="AH146" s="21"/>
-      <x:c r="AI146"/>
+      <x:c r="AI146" s="21"/>
     </x:row>
     <x:row r="147" ht="23" customHeight="1">
       <x:c r="A147" s="21"/>
@@ -5905,7 +5798,7 @@
       <x:c r="G147" s="21"/>
       <x:c r="H147" s="21"/>
       <x:c r="I147" s="21"/>
-      <x:c r="J147" s="28"/>
+      <x:c r="J147" s="21"/>
       <x:c r="K147" s="21"/>
       <x:c r="L147" s="21"/>
       <x:c r="M147" s="21"/>
@@ -5930,7 +5823,7 @@
       <x:c r="AF147" s="21"/>
       <x:c r="AG147" s="21"/>
       <x:c r="AH147" s="21"/>
-      <x:c r="AI147"/>
+      <x:c r="AI147" s="21"/>
     </x:row>
     <x:row r="148" ht="23" customHeight="1">
       <x:c r="A148" s="21"/>
@@ -5942,7 +5835,7 @@
       <x:c r="G148" s="21"/>
       <x:c r="H148" s="21"/>
       <x:c r="I148" s="21"/>
-      <x:c r="J148" s="28"/>
+      <x:c r="J148" s="21"/>
       <x:c r="K148" s="21"/>
       <x:c r="L148" s="21"/>
       <x:c r="M148" s="21"/>
@@ -5967,7 +5860,7 @@
       <x:c r="AF148" s="21"/>
       <x:c r="AG148" s="21"/>
       <x:c r="AH148" s="21"/>
-      <x:c r="AI148"/>
+      <x:c r="AI148" s="21"/>
     </x:row>
     <x:row r="149" ht="23" customHeight="1">
       <x:c r="A149" s="21"/>
@@ -5979,7 +5872,7 @@
       <x:c r="G149" s="21"/>
       <x:c r="H149" s="21"/>
       <x:c r="I149" s="21"/>
-      <x:c r="J149" s="28"/>
+      <x:c r="J149" s="21"/>
       <x:c r="K149" s="21"/>
       <x:c r="L149" s="21"/>
       <x:c r="M149" s="21"/>
@@ -6004,7 +5897,7 @@
       <x:c r="AF149" s="21"/>
       <x:c r="AG149" s="21"/>
       <x:c r="AH149" s="21"/>
-      <x:c r="AI149"/>
+      <x:c r="AI149" s="21"/>
     </x:row>
     <x:row r="150" ht="23" customHeight="1">
       <x:c r="A150" s="21"/>
@@ -6016,7 +5909,7 @@
       <x:c r="G150" s="21"/>
       <x:c r="H150" s="21"/>
       <x:c r="I150" s="21"/>
-      <x:c r="J150" s="28"/>
+      <x:c r="J150" s="21"/>
       <x:c r="K150" s="21"/>
       <x:c r="L150" s="21"/>
       <x:c r="M150" s="21"/>
@@ -6041,7 +5934,7 @@
       <x:c r="AF150" s="21"/>
       <x:c r="AG150" s="21"/>
       <x:c r="AH150" s="21"/>
-      <x:c r="AI150"/>
+      <x:c r="AI150" s="21"/>
     </x:row>
     <x:row r="151" ht="23" customHeight="1">
       <x:c r="A151" s="21"/>
@@ -6053,7 +5946,7 @@
       <x:c r="G151" s="21"/>
       <x:c r="H151" s="21"/>
       <x:c r="I151" s="21"/>
-      <x:c r="J151" s="28"/>
+      <x:c r="J151" s="21"/>
       <x:c r="K151" s="21"/>
       <x:c r="L151" s="21"/>
       <x:c r="M151" s="21"/>
@@ -6078,7 +5971,7 @@
       <x:c r="AF151" s="21"/>
       <x:c r="AG151" s="21"/>
       <x:c r="AH151" s="21"/>
-      <x:c r="AI151"/>
+      <x:c r="AI151" s="21"/>
     </x:row>
     <x:row r="152" ht="23" customHeight="1">
       <x:c r="A152" s="21"/>
@@ -6090,7 +5983,7 @@
       <x:c r="G152" s="21"/>
       <x:c r="H152" s="21"/>
       <x:c r="I152" s="21"/>
-      <x:c r="J152" s="28"/>
+      <x:c r="J152" s="21"/>
       <x:c r="K152" s="21"/>
       <x:c r="L152" s="21"/>
       <x:c r="M152" s="21"/>
@@ -6115,7 +6008,7 @@
       <x:c r="AF152" s="21"/>
       <x:c r="AG152" s="21"/>
       <x:c r="AH152" s="21"/>
-      <x:c r="AI152"/>
+      <x:c r="AI152" s="21"/>
     </x:row>
     <x:row r="153" ht="23" customHeight="1">
       <x:c r="A153" s="21"/>
@@ -6127,7 +6020,7 @@
       <x:c r="G153" s="21"/>
       <x:c r="H153" s="21"/>
       <x:c r="I153" s="21"/>
-      <x:c r="J153" s="28"/>
+      <x:c r="J153" s="21"/>
       <x:c r="K153" s="21"/>
       <x:c r="L153" s="21"/>
       <x:c r="M153" s="21"/>
@@ -6152,7 +6045,7 @@
       <x:c r="AF153" s="21"/>
       <x:c r="AG153" s="21"/>
       <x:c r="AH153" s="21"/>
-      <x:c r="AI153"/>
+      <x:c r="AI153" s="21"/>
     </x:row>
     <x:row r="154" ht="23" customHeight="1">
       <x:c r="A154" s="21"/>
@@ -6164,7 +6057,7 @@
       <x:c r="G154" s="21"/>
       <x:c r="H154" s="21"/>
       <x:c r="I154" s="21"/>
-      <x:c r="J154" s="28"/>
+      <x:c r="J154" s="21"/>
       <x:c r="K154" s="21"/>
       <x:c r="L154" s="21"/>
       <x:c r="M154" s="21"/>
@@ -6189,7 +6082,7 @@
       <x:c r="AF154" s="21"/>
       <x:c r="AG154" s="21"/>
       <x:c r="AH154" s="21"/>
-      <x:c r="AI154"/>
+      <x:c r="AI154" s="21"/>
     </x:row>
     <x:row r="155" ht="23" customHeight="1">
       <x:c r="A155" s="21"/>
@@ -6201,7 +6094,7 @@
       <x:c r="G155" s="21"/>
       <x:c r="H155" s="21"/>
       <x:c r="I155" s="21"/>
-      <x:c r="J155" s="28"/>
+      <x:c r="J155" s="21"/>
       <x:c r="K155" s="21"/>
       <x:c r="L155" s="21"/>
       <x:c r="M155" s="21"/>
@@ -6226,7 +6119,7 @@
       <x:c r="AF155" s="21"/>
       <x:c r="AG155" s="21"/>
       <x:c r="AH155" s="21"/>
-      <x:c r="AI155"/>
+      <x:c r="AI155" s="21"/>
     </x:row>
     <x:row r="156" ht="23" customHeight="1">
       <x:c r="A156" s="21"/>
@@ -6238,7 +6131,7 @@
       <x:c r="G156" s="21"/>
       <x:c r="H156" s="21"/>
       <x:c r="I156" s="21"/>
-      <x:c r="J156" s="28"/>
+      <x:c r="J156" s="21"/>
       <x:c r="K156" s="21"/>
       <x:c r="L156" s="21"/>
       <x:c r="M156" s="21"/>
@@ -6263,7 +6156,7 @@
       <x:c r="AF156" s="21"/>
       <x:c r="AG156" s="21"/>
       <x:c r="AH156" s="21"/>
-      <x:c r="AI156"/>
+      <x:c r="AI156" s="21"/>
     </x:row>
     <x:row r="157" ht="23" customHeight="1">
       <x:c r="A157" s="21"/>
@@ -6275,7 +6168,7 @@
       <x:c r="G157" s="21"/>
       <x:c r="H157" s="21"/>
       <x:c r="I157" s="21"/>
-      <x:c r="J157" s="28"/>
+      <x:c r="J157" s="21"/>
       <x:c r="K157" s="21"/>
       <x:c r="L157" s="21"/>
       <x:c r="M157" s="21"/>
@@ -6300,7 +6193,7 @@
       <x:c r="AF157" s="21"/>
       <x:c r="AG157" s="21"/>
       <x:c r="AH157" s="21"/>
-      <x:c r="AI157"/>
+      <x:c r="AI157" s="21"/>
     </x:row>
     <x:row r="158" ht="23" customHeight="1">
       <x:c r="A158" s="21"/>
@@ -6312,7 +6205,7 @@
       <x:c r="G158" s="21"/>
       <x:c r="H158" s="21"/>
       <x:c r="I158" s="21"/>
-      <x:c r="J158" s="28"/>
+      <x:c r="J158" s="21"/>
       <x:c r="K158" s="21"/>
       <x:c r="L158" s="21"/>
       <x:c r="M158" s="21"/>
@@ -6337,7 +6230,7 @@
       <x:c r="AF158" s="21"/>
       <x:c r="AG158" s="21"/>
       <x:c r="AH158" s="21"/>
-      <x:c r="AI158"/>
+      <x:c r="AI158" s="21"/>
     </x:row>
     <x:row r="159" ht="23" customHeight="1">
       <x:c r="A159" s="21"/>
@@ -6349,7 +6242,7 @@
       <x:c r="G159" s="21"/>
       <x:c r="H159" s="21"/>
       <x:c r="I159" s="21"/>
-      <x:c r="J159" s="28"/>
+      <x:c r="J159" s="21"/>
       <x:c r="K159" s="21"/>
       <x:c r="L159" s="21"/>
       <x:c r="M159" s="21"/>
@@ -6374,7 +6267,7 @@
       <x:c r="AF159" s="21"/>
       <x:c r="AG159" s="21"/>
       <x:c r="AH159" s="21"/>
-      <x:c r="AI159"/>
+      <x:c r="AI159" s="21"/>
     </x:row>
     <x:row r="160" ht="23" customHeight="1">
       <x:c r="A160" s="21"/>
@@ -6386,7 +6279,7 @@
       <x:c r="G160" s="21"/>
       <x:c r="H160" s="21"/>
       <x:c r="I160" s="21"/>
-      <x:c r="J160" s="28"/>
+      <x:c r="J160" s="21"/>
       <x:c r="K160" s="21"/>
       <x:c r="L160" s="21"/>
       <x:c r="M160" s="21"/>
@@ -6411,7 +6304,7 @@
       <x:c r="AF160" s="21"/>
       <x:c r="AG160" s="21"/>
       <x:c r="AH160" s="21"/>
-      <x:c r="AI160"/>
+      <x:c r="AI160" s="21"/>
     </x:row>
     <x:row r="161" ht="23" customHeight="1">
       <x:c r="A161" s="21"/>
@@ -6423,7 +6316,7 @@
       <x:c r="G161" s="21"/>
       <x:c r="H161" s="21"/>
       <x:c r="I161" s="21"/>
-      <x:c r="J161" s="28"/>
+      <x:c r="J161" s="21"/>
       <x:c r="K161" s="21"/>
       <x:c r="L161" s="21"/>
       <x:c r="M161" s="21"/>
@@ -6448,7 +6341,7 @@
       <x:c r="AF161" s="21"/>
       <x:c r="AG161" s="21"/>
       <x:c r="AH161" s="21"/>
-      <x:c r="AI161"/>
+      <x:c r="AI161" s="21"/>
     </x:row>
     <x:row r="162" ht="23" customHeight="1">
       <x:c r="A162" s="21"/>
@@ -6460,7 +6353,7 @@
       <x:c r="G162" s="21"/>
       <x:c r="H162" s="21"/>
       <x:c r="I162" s="21"/>
-      <x:c r="J162" s="28"/>
+      <x:c r="J162" s="21"/>
       <x:c r="K162" s="21"/>
       <x:c r="L162" s="21"/>
       <x:c r="M162" s="21"/>
@@ -6485,7 +6378,7 @@
       <x:c r="AF162" s="21"/>
       <x:c r="AG162" s="21"/>
       <x:c r="AH162" s="21"/>
-      <x:c r="AI162"/>
+      <x:c r="AI162" s="21"/>
     </x:row>
     <x:row r="163" ht="23" customHeight="1">
       <x:c r="A163" s="21"/>
@@ -6497,7 +6390,7 @@
       <x:c r="G163" s="21"/>
       <x:c r="H163" s="21"/>
       <x:c r="I163" s="21"/>
-      <x:c r="J163" s="28"/>
+      <x:c r="J163" s="21"/>
       <x:c r="K163" s="21"/>
       <x:c r="L163" s="21"/>
       <x:c r="M163" s="21"/>
@@ -6522,7 +6415,7 @@
       <x:c r="AF163" s="21"/>
       <x:c r="AG163" s="21"/>
       <x:c r="AH163" s="21"/>
-      <x:c r="AI163"/>
+      <x:c r="AI163" s="21"/>
     </x:row>
     <x:row r="164" ht="23" customHeight="1">
       <x:c r="A164" s="21"/>
@@ -6534,7 +6427,7 @@
       <x:c r="G164" s="21"/>
       <x:c r="H164" s="21"/>
       <x:c r="I164" s="21"/>
-      <x:c r="J164" s="28"/>
+      <x:c r="J164" s="21"/>
       <x:c r="K164" s="21"/>
       <x:c r="L164" s="21"/>
       <x:c r="M164" s="21"/>
@@ -6559,7 +6452,7 @@
       <x:c r="AF164" s="21"/>
       <x:c r="AG164" s="21"/>
       <x:c r="AH164" s="21"/>
-      <x:c r="AI164"/>
+      <x:c r="AI164" s="21"/>
     </x:row>
     <x:row r="165" ht="23" customHeight="1">
       <x:c r="A165" s="21"/>
@@ -6571,7 +6464,7 @@
       <x:c r="G165" s="21"/>
       <x:c r="H165" s="21"/>
       <x:c r="I165" s="21"/>
-      <x:c r="J165" s="28"/>
+      <x:c r="J165" s="21"/>
       <x:c r="K165" s="21"/>
       <x:c r="L165" s="21"/>
       <x:c r="M165" s="21"/>
@@ -6596,7 +6489,7 @@
       <x:c r="AF165" s="21"/>
       <x:c r="AG165" s="21"/>
       <x:c r="AH165" s="21"/>
-      <x:c r="AI165"/>
+      <x:c r="AI165" s="21"/>
     </x:row>
     <x:row r="166" ht="23" customHeight="1">
       <x:c r="A166" s="21"/>
@@ -6608,7 +6501,7 @@
       <x:c r="G166" s="21"/>
       <x:c r="H166" s="21"/>
       <x:c r="I166" s="21"/>
-      <x:c r="J166" s="28"/>
+      <x:c r="J166" s="21"/>
       <x:c r="K166" s="21"/>
       <x:c r="L166" s="21"/>
       <x:c r="M166" s="21"/>
@@ -6633,7 +6526,7 @@
       <x:c r="AF166" s="21"/>
       <x:c r="AG166" s="21"/>
       <x:c r="AH166" s="21"/>
-      <x:c r="AI166"/>
+      <x:c r="AI166" s="21"/>
     </x:row>
     <x:row r="167" ht="23" customHeight="1">
       <x:c r="A167" s="21"/>
@@ -6645,7 +6538,7 @@
       <x:c r="G167" s="21"/>
       <x:c r="H167" s="21"/>
       <x:c r="I167" s="21"/>
-      <x:c r="J167" s="28"/>
+      <x:c r="J167" s="21"/>
       <x:c r="K167" s="21"/>
       <x:c r="L167" s="21"/>
       <x:c r="M167" s="21"/>
@@ -6670,7 +6563,7 @@
       <x:c r="AF167" s="21"/>
       <x:c r="AG167" s="21"/>
       <x:c r="AH167" s="21"/>
-      <x:c r="AI167"/>
+      <x:c r="AI167" s="21"/>
     </x:row>
     <x:row r="168" ht="23" customHeight="1">
       <x:c r="A168" s="21"/>
@@ -6682,7 +6575,7 @@
       <x:c r="G168" s="21"/>
       <x:c r="H168" s="21"/>
       <x:c r="I168" s="21"/>
-      <x:c r="J168" s="28"/>
+      <x:c r="J168" s="21"/>
       <x:c r="K168" s="21"/>
       <x:c r="L168" s="21"/>
       <x:c r="M168" s="21"/>
@@ -6707,7 +6600,7 @@
       <x:c r="AF168" s="21"/>
       <x:c r="AG168" s="21"/>
       <x:c r="AH168" s="21"/>
-      <x:c r="AI168"/>
+      <x:c r="AI168" s="21"/>
     </x:row>
     <x:row r="169" ht="23" customHeight="1">
       <x:c r="A169" s="21"/>
@@ -6719,7 +6612,7 @@
       <x:c r="G169" s="21"/>
       <x:c r="H169" s="21"/>
       <x:c r="I169" s="21"/>
-      <x:c r="J169" s="28"/>
+      <x:c r="J169" s="21"/>
       <x:c r="K169" s="21"/>
       <x:c r="L169" s="21"/>
       <x:c r="M169" s="21"/>
@@ -6744,7 +6637,7 @@
       <x:c r="AF169" s="21"/>
       <x:c r="AG169" s="21"/>
       <x:c r="AH169" s="21"/>
-      <x:c r="AI169"/>
+      <x:c r="AI169" s="21"/>
     </x:row>
     <x:row r="170" ht="23" customHeight="1">
       <x:c r="A170" s="21"/>
@@ -6756,7 +6649,7 @@
       <x:c r="G170" s="21"/>
       <x:c r="H170" s="21"/>
       <x:c r="I170" s="21"/>
-      <x:c r="J170" s="28"/>
+      <x:c r="J170" s="21"/>
       <x:c r="K170" s="21"/>
       <x:c r="L170" s="21"/>
       <x:c r="M170" s="21"/>
@@ -6781,7 +6674,7 @@
       <x:c r="AF170" s="21"/>
       <x:c r="AG170" s="21"/>
       <x:c r="AH170" s="21"/>
-      <x:c r="AI170"/>
+      <x:c r="AI170" s="21"/>
     </x:row>
     <x:row r="171" ht="23" customHeight="1">
       <x:c r="A171" s="21"/>
@@ -6793,7 +6686,7 @@
       <x:c r="G171" s="21"/>
       <x:c r="H171" s="21"/>
       <x:c r="I171" s="21"/>
-      <x:c r="J171" s="28"/>
+      <x:c r="J171" s="21"/>
       <x:c r="K171" s="21"/>
       <x:c r="L171" s="21"/>
       <x:c r="M171" s="21"/>
@@ -6818,7 +6711,7 @@
       <x:c r="AF171" s="21"/>
       <x:c r="AG171" s="21"/>
       <x:c r="AH171" s="21"/>
-      <x:c r="AI171"/>
+      <x:c r="AI171" s="21"/>
     </x:row>
     <x:row r="172" ht="23" customHeight="1">
       <x:c r="A172" s="21"/>
@@ -6830,7 +6723,7 @@
       <x:c r="G172" s="21"/>
       <x:c r="H172" s="21"/>
       <x:c r="I172" s="21"/>
-      <x:c r="J172" s="28"/>
+      <x:c r="J172" s="21"/>
       <x:c r="K172" s="21"/>
       <x:c r="L172" s="21"/>
       <x:c r="M172" s="21"/>
@@ -6855,7 +6748,7 @@
       <x:c r="AF172" s="21"/>
       <x:c r="AG172" s="21"/>
       <x:c r="AH172" s="21"/>
-      <x:c r="AI172"/>
+      <x:c r="AI172" s="21"/>
     </x:row>
     <x:row r="173" ht="23" customHeight="1">
       <x:c r="A173" s="21"/>
@@ -6867,7 +6760,7 @@
       <x:c r="G173" s="21"/>
       <x:c r="H173" s="21"/>
       <x:c r="I173" s="21"/>
-      <x:c r="J173" s="28"/>
+      <x:c r="J173" s="21"/>
       <x:c r="K173" s="21"/>
       <x:c r="L173" s="21"/>
       <x:c r="M173" s="21"/>
@@ -6892,7 +6785,7 @@
       <x:c r="AF173" s="21"/>
       <x:c r="AG173" s="21"/>
       <x:c r="AH173" s="21"/>
-      <x:c r="AI173"/>
+      <x:c r="AI173" s="21"/>
     </x:row>
     <x:row r="174" ht="23" customHeight="1">
       <x:c r="A174" s="21"/>
@@ -6904,7 +6797,7 @@
       <x:c r="G174" s="21"/>
       <x:c r="H174" s="21"/>
       <x:c r="I174" s="21"/>
-      <x:c r="J174" s="28"/>
+      <x:c r="J174" s="21"/>
       <x:c r="K174" s="21"/>
       <x:c r="L174" s="21"/>
       <x:c r="M174" s="21"/>
@@ -6929,7 +6822,7 @@
       <x:c r="AF174" s="21"/>
       <x:c r="AG174" s="21"/>
       <x:c r="AH174" s="21"/>
-      <x:c r="AI174"/>
+      <x:c r="AI174" s="21"/>
     </x:row>
     <x:row r="175" ht="23" customHeight="1">
       <x:c r="A175" s="21"/>
@@ -6941,7 +6834,7 @@
       <x:c r="G175" s="21"/>
       <x:c r="H175" s="21"/>
       <x:c r="I175" s="21"/>
-      <x:c r="J175" s="28"/>
+      <x:c r="J175" s="21"/>
       <x:c r="K175" s="21"/>
       <x:c r="L175" s="21"/>
       <x:c r="M175" s="21"/>
@@ -6966,7 +6859,7 @@
       <x:c r="AF175" s="21"/>
       <x:c r="AG175" s="21"/>
       <x:c r="AH175" s="21"/>
-      <x:c r="AI175"/>
+      <x:c r="AI175" s="21"/>
     </x:row>
     <x:row r="176" ht="23" customHeight="1">
       <x:c r="A176" s="21"/>
@@ -6978,7 +6871,7 @@
       <x:c r="G176" s="21"/>
       <x:c r="H176" s="21"/>
       <x:c r="I176" s="21"/>
-      <x:c r="J176" s="28"/>
+      <x:c r="J176" s="21"/>
       <x:c r="K176" s="21"/>
       <x:c r="L176" s="21"/>
       <x:c r="M176" s="21"/>
@@ -7003,7 +6896,7 @@
       <x:c r="AF176" s="21"/>
       <x:c r="AG176" s="21"/>
       <x:c r="AH176" s="21"/>
-      <x:c r="AI176"/>
+      <x:c r="AI176" s="21"/>
     </x:row>
     <x:row r="177" ht="23" customHeight="1">
       <x:c r="A177" s="21"/>
@@ -7015,7 +6908,7 @@
       <x:c r="G177" s="21"/>
       <x:c r="H177" s="21"/>
       <x:c r="I177" s="21"/>
-      <x:c r="J177" s="28"/>
+      <x:c r="J177" s="21"/>
       <x:c r="K177" s="21"/>
       <x:c r="L177" s="21"/>
       <x:c r="M177" s="21"/>
@@ -7040,7 +6933,7 @@
       <x:c r="AF177" s="21"/>
       <x:c r="AG177" s="21"/>
       <x:c r="AH177" s="21"/>
-      <x:c r="AI177"/>
+      <x:c r="AI177" s="21"/>
     </x:row>
     <x:row r="178" ht="23" customHeight="1">
       <x:c r="A178" s="21"/>
@@ -7052,7 +6945,7 @@
       <x:c r="G178" s="21"/>
       <x:c r="H178" s="21"/>
       <x:c r="I178" s="21"/>
-      <x:c r="J178" s="28"/>
+      <x:c r="J178" s="21"/>
       <x:c r="K178" s="21"/>
       <x:c r="L178" s="21"/>
       <x:c r="M178" s="21"/>
@@ -7077,7 +6970,7 @@
       <x:c r="AF178" s="21"/>
       <x:c r="AG178" s="21"/>
       <x:c r="AH178" s="21"/>
-      <x:c r="AI178"/>
+      <x:c r="AI178" s="21"/>
     </x:row>
     <x:row r="179" ht="23" customHeight="1">
       <x:c r="A179" s="21"/>
@@ -7089,7 +6982,7 @@
       <x:c r="G179" s="21"/>
       <x:c r="H179" s="21"/>
       <x:c r="I179" s="21"/>
-      <x:c r="J179" s="28"/>
+      <x:c r="J179" s="21"/>
       <x:c r="K179" s="21"/>
       <x:c r="L179" s="21"/>
       <x:c r="M179" s="21"/>
@@ -7114,7 +7007,7 @@
       <x:c r="AF179" s="21"/>
       <x:c r="AG179" s="21"/>
       <x:c r="AH179" s="21"/>
-      <x:c r="AI179"/>
+      <x:c r="AI179" s="21"/>
     </x:row>
     <x:row r="180" ht="23" customHeight="1">
       <x:c r="A180" s="21"/>
@@ -7126,7 +7019,7 @@
       <x:c r="G180" s="21"/>
       <x:c r="H180" s="21"/>
       <x:c r="I180" s="21"/>
-      <x:c r="J180" s="28"/>
+      <x:c r="J180" s="21"/>
       <x:c r="K180" s="21"/>
       <x:c r="L180" s="21"/>
       <x:c r="M180" s="21"/>
@@ -7151,7 +7044,7 @@
       <x:c r="AF180" s="21"/>
       <x:c r="AG180" s="21"/>
       <x:c r="AH180" s="21"/>
-      <x:c r="AI180"/>
+      <x:c r="AI180" s="21"/>
     </x:row>
     <x:row r="181" ht="23" customHeight="1">
       <x:c r="A181" s="21"/>
@@ -7163,7 +7056,7 @@
       <x:c r="G181" s="21"/>
       <x:c r="H181" s="21"/>
       <x:c r="I181" s="21"/>
-      <x:c r="J181" s="28"/>
+      <x:c r="J181" s="21"/>
       <x:c r="K181" s="21"/>
       <x:c r="L181" s="21"/>
       <x:c r="M181" s="21"/>
@@ -7188,7 +7081,7 @@
       <x:c r="AF181" s="21"/>
       <x:c r="AG181" s="21"/>
       <x:c r="AH181" s="21"/>
-      <x:c r="AI181"/>
+      <x:c r="AI181" s="21"/>
     </x:row>
     <x:row r="182" ht="23" customHeight="1">
       <x:c r="A182" s="21"/>
@@ -7200,7 +7093,7 @@
       <x:c r="G182" s="21"/>
       <x:c r="H182" s="21"/>
       <x:c r="I182" s="21"/>
-      <x:c r="J182" s="28"/>
+      <x:c r="J182" s="21"/>
       <x:c r="K182" s="21"/>
       <x:c r="L182" s="21"/>
       <x:c r="M182" s="21"/>
@@ -7225,7 +7118,7 @@
       <x:c r="AF182" s="21"/>
       <x:c r="AG182" s="21"/>
       <x:c r="AH182" s="21"/>
-      <x:c r="AI182"/>
+      <x:c r="AI182" s="21"/>
     </x:row>
     <x:row r="183" ht="23" customHeight="1">
       <x:c r="A183" s="21"/>
@@ -7237,7 +7130,7 @@
       <x:c r="G183" s="21"/>
       <x:c r="H183" s="21"/>
       <x:c r="I183" s="21"/>
-      <x:c r="J183" s="28"/>
+      <x:c r="J183" s="21"/>
       <x:c r="K183" s="21"/>
       <x:c r="L183" s="21"/>
       <x:c r="M183" s="21"/>
@@ -7262,7 +7155,7 @@
       <x:c r="AF183" s="21"/>
       <x:c r="AG183" s="21"/>
       <x:c r="AH183" s="21"/>
-      <x:c r="AI183"/>
+      <x:c r="AI183" s="21"/>
     </x:row>
     <x:row r="184" ht="23" customHeight="1">
       <x:c r="A184" s="21"/>
@@ -7274,7 +7167,7 @@
       <x:c r="G184" s="21"/>
       <x:c r="H184" s="21"/>
       <x:c r="I184" s="21"/>
-      <x:c r="J184" s="28"/>
+      <x:c r="J184" s="21"/>
       <x:c r="K184" s="21"/>
       <x:c r="L184" s="21"/>
       <x:c r="M184" s="21"/>
@@ -7299,7 +7192,7 @@
       <x:c r="AF184" s="21"/>
       <x:c r="AG184" s="21"/>
       <x:c r="AH184" s="21"/>
-      <x:c r="AI184"/>
+      <x:c r="AI184" s="21"/>
     </x:row>
     <x:row r="185" ht="23" customHeight="1">
       <x:c r="A185" s="21"/>
@@ -7311,7 +7204,7 @@
       <x:c r="G185" s="21"/>
       <x:c r="H185" s="21"/>
       <x:c r="I185" s="21"/>
-      <x:c r="J185" s="28"/>
+      <x:c r="J185" s="21"/>
       <x:c r="K185" s="21"/>
       <x:c r="L185" s="21"/>
       <x:c r="M185" s="21"/>
@@ -7336,7 +7229,7 @@
       <x:c r="AF185" s="21"/>
       <x:c r="AG185" s="21"/>
       <x:c r="AH185" s="21"/>
-      <x:c r="AI185"/>
+      <x:c r="AI185" s="21"/>
     </x:row>
     <x:row r="186" ht="23" customHeight="1">
       <x:c r="A186" s="21"/>
@@ -7348,7 +7241,7 @@
       <x:c r="G186" s="21"/>
       <x:c r="H186" s="21"/>
       <x:c r="I186" s="21"/>
-      <x:c r="J186" s="28"/>
+      <x:c r="J186" s="21"/>
       <x:c r="K186" s="21"/>
       <x:c r="L186" s="21"/>
       <x:c r="M186" s="21"/>
@@ -7373,7 +7266,7 @@
       <x:c r="AF186" s="21"/>
       <x:c r="AG186" s="21"/>
       <x:c r="AH186" s="21"/>
-      <x:c r="AI186"/>
+      <x:c r="AI186" s="21"/>
     </x:row>
     <x:row r="187" ht="23" customHeight="1">
       <x:c r="A187" s="21"/>
@@ -7385,7 +7278,7 @@
       <x:c r="G187" s="21"/>
       <x:c r="H187" s="21"/>
       <x:c r="I187" s="21"/>
-      <x:c r="J187" s="28"/>
+      <x:c r="J187" s="21"/>
       <x:c r="K187" s="21"/>
       <x:c r="L187" s="21"/>
       <x:c r="M187" s="21"/>
@@ -7410,7 +7303,7 @@
       <x:c r="AF187" s="21"/>
       <x:c r="AG187" s="21"/>
       <x:c r="AH187" s="21"/>
-      <x:c r="AI187"/>
+      <x:c r="AI187" s="21"/>
     </x:row>
     <x:row r="188" ht="23" customHeight="1">
       <x:c r="A188" s="21"/>
@@ -7422,7 +7315,7 @@
       <x:c r="G188" s="21"/>
       <x:c r="H188" s="21"/>
       <x:c r="I188" s="21"/>
-      <x:c r="J188" s="28"/>
+      <x:c r="J188" s="21"/>
       <x:c r="K188" s="21"/>
       <x:c r="L188" s="21"/>
       <x:c r="M188" s="21"/>
@@ -7447,7 +7340,7 @@
       <x:c r="AF188" s="21"/>
       <x:c r="AG188" s="21"/>
       <x:c r="AH188" s="21"/>
-      <x:c r="AI188"/>
+      <x:c r="AI188" s="21"/>
     </x:row>
     <x:row r="189" ht="23" customHeight="1">
       <x:c r="A189" s="21"/>
@@ -7459,7 +7352,7 @@
       <x:c r="G189" s="21"/>
       <x:c r="H189" s="21"/>
       <x:c r="I189" s="21"/>
-      <x:c r="J189" s="28"/>
+      <x:c r="J189" s="21"/>
       <x:c r="K189" s="21"/>
       <x:c r="L189" s="21"/>
       <x:c r="M189" s="21"/>
@@ -7484,7 +7377,7 @@
       <x:c r="AF189" s="21"/>
       <x:c r="AG189" s="21"/>
       <x:c r="AH189" s="21"/>
-      <x:c r="AI189"/>
+      <x:c r="AI189" s="21"/>
     </x:row>
     <x:row r="190" ht="23" customHeight="1">
       <x:c r="A190" s="21"/>
@@ -7496,7 +7389,7 @@
       <x:c r="G190" s="21"/>
       <x:c r="H190" s="21"/>
       <x:c r="I190" s="21"/>
-      <x:c r="J190" s="28"/>
+      <x:c r="J190" s="21"/>
       <x:c r="K190" s="21"/>
       <x:c r="L190" s="21"/>
       <x:c r="M190" s="21"/>
@@ -7521,7 +7414,7 @@
       <x:c r="AF190" s="21"/>
       <x:c r="AG190" s="21"/>
       <x:c r="AH190" s="21"/>
-      <x:c r="AI190"/>
+      <x:c r="AI190" s="21"/>
     </x:row>
     <x:row r="191" ht="23" customHeight="1">
       <x:c r="A191" s="21"/>
@@ -7533,7 +7426,7 @@
       <x:c r="G191" s="21"/>
       <x:c r="H191" s="21"/>
       <x:c r="I191" s="21"/>
-      <x:c r="J191" s="28"/>
+      <x:c r="J191" s="21"/>
       <x:c r="K191" s="21"/>
       <x:c r="L191" s="21"/>
       <x:c r="M191" s="21"/>
@@ -7558,7 +7451,7 @@
       <x:c r="AF191" s="21"/>
       <x:c r="AG191" s="21"/>
       <x:c r="AH191" s="21"/>
-      <x:c r="AI191"/>
+      <x:c r="AI191" s="21"/>
     </x:row>
     <x:row r="192" ht="23" customHeight="1">
       <x:c r="A192" s="21"/>
@@ -7570,7 +7463,7 @@
       <x:c r="G192" s="21"/>
       <x:c r="H192" s="21"/>
       <x:c r="I192" s="21"/>
-      <x:c r="J192" s="28"/>
+      <x:c r="J192" s="21"/>
       <x:c r="K192" s="21"/>
       <x:c r="L192" s="21"/>
       <x:c r="M192" s="21"/>
@@ -7595,7 +7488,7 @@
       <x:c r="AF192" s="21"/>
       <x:c r="AG192" s="21"/>
       <x:c r="AH192" s="21"/>
-      <x:c r="AI192"/>
+      <x:c r="AI192" s="21"/>
     </x:row>
     <x:row r="193" ht="23" customHeight="1">
       <x:c r="A193" s="21"/>
@@ -7607,7 +7500,7 @@
       <x:c r="G193" s="21"/>
       <x:c r="H193" s="21"/>
       <x:c r="I193" s="21"/>
-      <x:c r="J193" s="28"/>
+      <x:c r="J193" s="21"/>
       <x:c r="K193" s="21"/>
       <x:c r="L193" s="21"/>
       <x:c r="M193" s="21"/>
@@ -7632,7 +7525,7 @@
       <x:c r="AF193" s="21"/>
       <x:c r="AG193" s="21"/>
       <x:c r="AH193" s="21"/>
-      <x:c r="AI193"/>
+      <x:c r="AI193" s="21"/>
     </x:row>
     <x:row r="194" ht="23" customHeight="1">
       <x:c r="A194" s="21"/>
@@ -7644,7 +7537,7 @@
       <x:c r="G194" s="21"/>
       <x:c r="H194" s="21"/>
       <x:c r="I194" s="21"/>
-      <x:c r="J194" s="28"/>
+      <x:c r="J194" s="21"/>
       <x:c r="K194" s="21"/>
       <x:c r="L194" s="21"/>
       <x:c r="M194" s="21"/>
@@ -7669,7 +7562,7 @@
       <x:c r="AF194" s="21"/>
       <x:c r="AG194" s="21"/>
       <x:c r="AH194" s="21"/>
-      <x:c r="AI194"/>
+      <x:c r="AI194" s="21"/>
     </x:row>
     <x:row r="195" ht="23" customHeight="1">
       <x:c r="A195" s="21"/>
@@ -7681,7 +7574,7 @@
       <x:c r="G195" s="21"/>
       <x:c r="H195" s="21"/>
       <x:c r="I195" s="21"/>
-      <x:c r="J195" s="28"/>
+      <x:c r="J195" s="21"/>
       <x:c r="K195" s="21"/>
       <x:c r="L195" s="21"/>
       <x:c r="M195" s="21"/>
@@ -7706,7 +7599,7 @@
       <x:c r="AF195" s="21"/>
       <x:c r="AG195" s="21"/>
       <x:c r="AH195" s="21"/>
-      <x:c r="AI195"/>
+      <x:c r="AI195" s="21"/>
     </x:row>
     <x:row r="196" ht="23" customHeight="1">
       <x:c r="A196" s="21"/>
@@ -7718,7 +7611,7 @@
       <x:c r="G196" s="21"/>
       <x:c r="H196" s="21"/>
       <x:c r="I196" s="21"/>
-      <x:c r="J196" s="28"/>
+      <x:c r="J196" s="21"/>
       <x:c r="K196" s="21"/>
       <x:c r="L196" s="21"/>
       <x:c r="M196" s="21"/>
@@ -7743,7 +7636,7 @@
       <x:c r="AF196" s="21"/>
       <x:c r="AG196" s="21"/>
       <x:c r="AH196" s="21"/>
-      <x:c r="AI196"/>
+      <x:c r="AI196" s="21"/>
     </x:row>
     <x:row r="197" ht="23" customHeight="1">
       <x:c r="A197" s="21"/>
@@ -7755,7 +7648,7 @@
       <x:c r="G197" s="21"/>
       <x:c r="H197" s="21"/>
       <x:c r="I197" s="21"/>
-      <x:c r="J197" s="28"/>
+      <x:c r="J197" s="21"/>
       <x:c r="K197" s="21"/>
       <x:c r="L197" s="21"/>
       <x:c r="M197" s="21"/>
@@ -7780,7 +7673,7 @@
       <x:c r="AF197" s="21"/>
       <x:c r="AG197" s="21"/>
       <x:c r="AH197" s="21"/>
-      <x:c r="AI197"/>
+      <x:c r="AI197" s="21"/>
     </x:row>
     <x:row r="198" ht="23" customHeight="1">
       <x:c r="A198" s="21"/>
@@ -7792,7 +7685,7 @@
       <x:c r="G198" s="21"/>
       <x:c r="H198" s="21"/>
       <x:c r="I198" s="21"/>
-      <x:c r="J198" s="28"/>
+      <x:c r="J198" s="21"/>
       <x:c r="K198" s="21"/>
       <x:c r="L198" s="21"/>
       <x:c r="M198" s="21"/>
@@ -7817,7 +7710,7 @@
       <x:c r="AF198" s="21"/>
       <x:c r="AG198" s="21"/>
       <x:c r="AH198" s="21"/>
-      <x:c r="AI198"/>
+      <x:c r="AI198" s="21"/>
     </x:row>
     <x:row r="199" ht="23" customHeight="1">
       <x:c r="A199" s="21"/>
@@ -7829,7 +7722,7 @@
       <x:c r="G199" s="21"/>
       <x:c r="H199" s="21"/>
       <x:c r="I199" s="21"/>
-      <x:c r="J199" s="28"/>
+      <x:c r="J199" s="21"/>
       <x:c r="K199" s="21"/>
       <x:c r="L199" s="21"/>
       <x:c r="M199" s="21"/>
@@ -7854,7 +7747,7 @@
       <x:c r="AF199" s="21"/>
       <x:c r="AG199" s="21"/>
       <x:c r="AH199" s="21"/>
-      <x:c r="AI199"/>
+      <x:c r="AI199" s="21"/>
     </x:row>
     <x:row r="200" ht="23" customHeight="1">
       <x:c r="A200" s="21"/>
@@ -7866,7 +7759,7 @@
       <x:c r="G200" s="21"/>
       <x:c r="H200" s="21"/>
       <x:c r="I200" s="21"/>
-      <x:c r="J200" s="28"/>
+      <x:c r="J200" s="21"/>
       <x:c r="K200" s="21"/>
       <x:c r="L200" s="21"/>
       <x:c r="M200" s="21"/>
@@ -7891,13 +7784,13 @@
       <x:c r="AF200" s="21"/>
       <x:c r="AG200" s="21"/>
       <x:c r="AH200" s="21"/>
-      <x:c r="AI200"/>
+      <x:c r="AI200" s="21"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:AH1"/>
-    <x:mergeCell ref="A2:AH2"/>
-    <x:mergeCell ref="A3:AH3"/>
+    <x:mergeCell ref="A1:AI1"/>
+    <x:mergeCell ref="A2:AI2"/>
+    <x:mergeCell ref="A3:AI3"/>
   </x:mergeCells>
   <x:dataValidations count="8">
     <x:dataValidation type="list" sqref="E5:E200">

</xml_diff>